<commit_message>
Primer avance del documento de TFC2
</commit_message>
<xml_diff>
--- a/REPORTES/Cronograma-MHinojosa.xlsx
+++ b/REPORTES/Cronograma-MHinojosa.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Desktop\TESIS 2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Desktop\TESIS 2\TFC2_20212123_MHinojosa\TFC2-20212123-LaTeX\REPORTES\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60F77230-AD9C-4396-8155-E9DDEE5CDFCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51195F97-3F79-41FA-944B-0DBD745DA4E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11310" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="75">
   <si>
     <t xml:space="preserve">Formulario: Cronograma de los trabajos y aplicación de entregables                                                        </t>
   </si>
@@ -206,9 +206,6 @@
     <t>Validación con mediciones empíricas</t>
   </si>
   <si>
-    <t>Manufactura de la PCB (envio desde China alrededor de 1 semana) - Prototipo</t>
-  </si>
-  <si>
     <t>Manufactura de la PCB - Diseño final</t>
   </si>
   <si>
@@ -261,6 +258,12 @@
   </si>
   <si>
     <t>AVANCE 3</t>
+  </si>
+  <si>
+    <t>Manufactura de la PCB  - Prototipo</t>
+  </si>
+  <si>
+    <t>Diagrama de flujo y lógica a seguir</t>
   </si>
 </sst>
 </file>
@@ -402,7 +405,7 @@
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="14">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -473,12 +476,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0"/>
-        <bgColor rgb="FFD9EAD3"/>
       </patternFill>
     </fill>
   </fills>
@@ -656,7 +653,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="76">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -804,29 +801,18 @@
     <xf numFmtId="9" fontId="21" fillId="7" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="19" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -847,14 +833,22 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1133,131 +1127,131 @@
     </row>
     <row r="2" spans="1:28" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
-      <c r="B2" s="62" t="s">
+      <c r="B2" s="61" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="63"/>
-      <c r="D2" s="63"/>
-      <c r="E2" s="63"/>
-      <c r="F2" s="63"/>
-      <c r="G2" s="63"/>
-      <c r="H2" s="63"/>
-      <c r="I2" s="63"/>
-      <c r="J2" s="63"/>
-      <c r="K2" s="63"/>
-      <c r="L2" s="64"/>
-      <c r="M2" s="63"/>
-      <c r="N2" s="63"/>
-      <c r="O2" s="63"/>
-      <c r="P2" s="63"/>
-      <c r="Q2" s="63"/>
-      <c r="R2" s="63"/>
-      <c r="S2" s="63"/>
-      <c r="T2" s="63"/>
-      <c r="U2" s="63"/>
-      <c r="V2" s="63"/>
-      <c r="W2" s="63"/>
-      <c r="X2" s="63"/>
-      <c r="Y2" s="63"/>
-      <c r="Z2" s="63"/>
-      <c r="AA2" s="63"/>
+      <c r="C2" s="62"/>
+      <c r="D2" s="62"/>
+      <c r="E2" s="62"/>
+      <c r="F2" s="62"/>
+      <c r="G2" s="62"/>
+      <c r="H2" s="62"/>
+      <c r="I2" s="62"/>
+      <c r="J2" s="62"/>
+      <c r="K2" s="62"/>
+      <c r="L2" s="63"/>
+      <c r="M2" s="62"/>
+      <c r="N2" s="62"/>
+      <c r="O2" s="62"/>
+      <c r="P2" s="62"/>
+      <c r="Q2" s="62"/>
+      <c r="R2" s="62"/>
+      <c r="S2" s="62"/>
+      <c r="T2" s="62"/>
+      <c r="U2" s="62"/>
+      <c r="V2" s="62"/>
+      <c r="W2" s="62"/>
+      <c r="X2" s="62"/>
+      <c r="Y2" s="62"/>
+      <c r="Z2" s="62"/>
+      <c r="AA2" s="62"/>
     </row>
     <row r="3" spans="1:28" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A3" s="3"/>
-      <c r="B3" s="65"/>
-      <c r="C3" s="66"/>
-      <c r="D3" s="67"/>
-      <c r="E3" s="66"/>
-      <c r="F3" s="66"/>
-      <c r="G3" s="66"/>
-      <c r="H3" s="66"/>
-      <c r="I3" s="66"/>
-      <c r="J3" s="66"/>
-      <c r="K3" s="66"/>
-      <c r="L3" s="68"/>
-      <c r="M3" s="66"/>
-      <c r="N3" s="66"/>
-      <c r="O3" s="66"/>
-      <c r="P3" s="66"/>
-      <c r="Q3" s="66"/>
-      <c r="R3" s="66"/>
-      <c r="S3" s="66"/>
-      <c r="T3" s="66"/>
-      <c r="U3" s="69"/>
-      <c r="V3" s="66"/>
-      <c r="W3" s="66"/>
-      <c r="X3" s="66"/>
-      <c r="Y3" s="66"/>
-      <c r="Z3" s="66"/>
-      <c r="AA3" s="66"/>
+      <c r="B3" s="64"/>
+      <c r="C3" s="65"/>
+      <c r="D3" s="66"/>
+      <c r="E3" s="65"/>
+      <c r="F3" s="65"/>
+      <c r="G3" s="65"/>
+      <c r="H3" s="65"/>
+      <c r="I3" s="65"/>
+      <c r="J3" s="65"/>
+      <c r="K3" s="65"/>
+      <c r="L3" s="67"/>
+      <c r="M3" s="65"/>
+      <c r="N3" s="65"/>
+      <c r="O3" s="65"/>
+      <c r="P3" s="65"/>
+      <c r="Q3" s="65"/>
+      <c r="R3" s="65"/>
+      <c r="S3" s="65"/>
+      <c r="T3" s="65"/>
+      <c r="U3" s="68"/>
+      <c r="V3" s="65"/>
+      <c r="W3" s="65"/>
+      <c r="X3" s="65"/>
+      <c r="Y3" s="65"/>
+      <c r="Z3" s="65"/>
+      <c r="AA3" s="65"/>
     </row>
     <row r="4" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="4"/>
-      <c r="B4" s="61" t="s">
+      <c r="B4" s="54" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="60"/>
-      <c r="D4" s="71" t="s">
+      <c r="C4" s="55"/>
+      <c r="D4" s="58" t="s">
         <v>33</v>
       </c>
-      <c r="E4" s="60"/>
-      <c r="F4" s="60"/>
-      <c r="G4" s="60"/>
-      <c r="H4" s="60"/>
+      <c r="E4" s="55"/>
+      <c r="F4" s="55"/>
+      <c r="G4" s="55"/>
+      <c r="H4" s="55"/>
       <c r="I4" s="5"/>
-      <c r="J4" s="61" t="s">
+      <c r="J4" s="54" t="s">
         <v>2</v>
       </c>
-      <c r="K4" s="60"/>
-      <c r="L4" s="70"/>
-      <c r="M4" s="60"/>
-      <c r="N4" s="60"/>
-      <c r="O4" s="60"/>
-      <c r="P4" s="60"/>
-      <c r="Q4" s="60"/>
-      <c r="R4" s="60"/>
-      <c r="S4" s="60"/>
-      <c r="T4" s="60"/>
-      <c r="U4" s="60"/>
-      <c r="V4" s="60"/>
-      <c r="W4" s="60"/>
-      <c r="X4" s="60"/>
+      <c r="K4" s="55"/>
+      <c r="L4" s="56"/>
+      <c r="M4" s="55"/>
+      <c r="N4" s="55"/>
+      <c r="O4" s="55"/>
+      <c r="P4" s="55"/>
+      <c r="Q4" s="55"/>
+      <c r="R4" s="55"/>
+      <c r="S4" s="55"/>
+      <c r="T4" s="55"/>
+      <c r="U4" s="55"/>
+      <c r="V4" s="55"/>
+      <c r="W4" s="55"/>
+      <c r="X4" s="55"/>
       <c r="Y4" s="6"/>
       <c r="Z4" s="6"/>
       <c r="AA4" s="6"/>
     </row>
     <row r="5" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="4"/>
-      <c r="B5" s="61" t="s">
+      <c r="B5" s="54" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="60"/>
-      <c r="D5" s="72" t="s">
+      <c r="C5" s="55"/>
+      <c r="D5" s="59" t="s">
         <v>34</v>
       </c>
-      <c r="E5" s="60"/>
-      <c r="F5" s="60"/>
-      <c r="G5" s="60"/>
-      <c r="H5" s="60"/>
+      <c r="E5" s="55"/>
+      <c r="F5" s="55"/>
+      <c r="G5" s="55"/>
+      <c r="H5" s="55"/>
       <c r="I5" s="8"/>
-      <c r="J5" s="73" t="s">
+      <c r="J5" s="60" t="s">
         <v>48</v>
       </c>
-      <c r="K5" s="60"/>
-      <c r="L5" s="59">
+      <c r="K5" s="55"/>
+      <c r="L5" s="57">
         <v>45991</v>
       </c>
-      <c r="M5" s="60"/>
-      <c r="N5" s="60"/>
-      <c r="O5" s="60"/>
-      <c r="P5" s="60"/>
-      <c r="Q5" s="60"/>
-      <c r="R5" s="60"/>
-      <c r="S5" s="60"/>
-      <c r="T5" s="60"/>
-      <c r="U5" s="60"/>
-      <c r="V5" s="60"/>
-      <c r="W5" s="60"/>
+      <c r="M5" s="55"/>
+      <c r="N5" s="55"/>
+      <c r="O5" s="55"/>
+      <c r="P5" s="55"/>
+      <c r="Q5" s="55"/>
+      <c r="R5" s="55"/>
+      <c r="S5" s="55"/>
+      <c r="T5" s="55"/>
+      <c r="U5" s="55"/>
+      <c r="V5" s="55"/>
+      <c r="W5" s="55"/>
       <c r="X5" s="9"/>
       <c r="Y5" s="9"/>
       <c r="Z5" s="9"/>
@@ -1265,24 +1259,24 @@
     </row>
     <row r="6" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="4"/>
-      <c r="B6" s="61" t="s">
+      <c r="B6" s="54" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="60"/>
-      <c r="D6" s="59">
+      <c r="C6" s="55"/>
+      <c r="D6" s="57">
         <v>45918</v>
       </c>
-      <c r="E6" s="60"/>
-      <c r="F6" s="60"/>
-      <c r="G6" s="60"/>
-      <c r="H6" s="60"/>
-      <c r="I6" s="60"/>
-      <c r="J6" s="60"/>
-      <c r="K6" s="60"/>
-      <c r="L6" s="60"/>
-      <c r="M6" s="60"/>
-      <c r="N6" s="60"/>
-      <c r="O6" s="60"/>
+      <c r="E6" s="55"/>
+      <c r="F6" s="55"/>
+      <c r="G6" s="55"/>
+      <c r="H6" s="55"/>
+      <c r="I6" s="55"/>
+      <c r="J6" s="55"/>
+      <c r="K6" s="55"/>
+      <c r="L6" s="55"/>
+      <c r="M6" s="55"/>
+      <c r="N6" s="55"/>
+      <c r="O6" s="55"/>
       <c r="P6" s="8"/>
       <c r="Q6" s="8"/>
       <c r="R6" s="8"/>
@@ -1329,34 +1323,34 @@
     </row>
     <row r="8" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="15"/>
-      <c r="B8" s="56" t="s">
+      <c r="B8" s="69" t="s">
         <v>35</v>
       </c>
-      <c r="C8" s="56" t="s">
+      <c r="C8" s="69" t="s">
         <v>21</v>
       </c>
-      <c r="D8" s="56" t="s">
+      <c r="D8" s="69" t="s">
         <v>22</v>
       </c>
-      <c r="E8" s="56" t="s">
+      <c r="E8" s="69" t="s">
         <v>23</v>
       </c>
-      <c r="F8" s="56" t="s">
+      <c r="F8" s="69" t="s">
         <v>24</v>
       </c>
-      <c r="G8" s="56" t="s">
+      <c r="G8" s="69" t="s">
         <v>25</v>
       </c>
-      <c r="H8" s="56" t="s">
+      <c r="H8" s="69" t="s">
         <v>26</v>
       </c>
-      <c r="I8" s="56" t="s">
+      <c r="I8" s="69" t="s">
         <v>27</v>
       </c>
-      <c r="J8" s="56" t="s">
+      <c r="J8" s="69" t="s">
         <v>28</v>
       </c>
-      <c r="K8" s="56" t="s">
+      <c r="K8" s="69" t="s">
         <v>29</v>
       </c>
       <c r="L8" s="16"/>
@@ -1379,16 +1373,16 @@
     </row>
     <row r="9" spans="1:28" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="17"/>
-      <c r="B9" s="56"/>
-      <c r="C9" s="56"/>
-      <c r="D9" s="56"/>
-      <c r="E9" s="56"/>
-      <c r="F9" s="56"/>
-      <c r="G9" s="56"/>
-      <c r="H9" s="56"/>
-      <c r="I9" s="56"/>
-      <c r="J9" s="56"/>
-      <c r="K9" s="56"/>
+      <c r="B9" s="69"/>
+      <c r="C9" s="69"/>
+      <c r="D9" s="69"/>
+      <c r="E9" s="69"/>
+      <c r="F9" s="69"/>
+      <c r="G9" s="69"/>
+      <c r="H9" s="69"/>
+      <c r="I9" s="69"/>
+      <c r="J9" s="69"/>
+      <c r="K9" s="69"/>
       <c r="L9" s="18" t="s">
         <v>5</v>
       </c>
@@ -1441,16 +1435,16 @@
     </row>
     <row r="10" spans="1:28" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="20"/>
-      <c r="B10" s="58"/>
-      <c r="C10" s="58"/>
-      <c r="D10" s="58"/>
-      <c r="E10" s="58"/>
-      <c r="F10" s="58"/>
-      <c r="G10" s="58"/>
-      <c r="H10" s="58"/>
-      <c r="I10" s="58"/>
-      <c r="J10" s="58"/>
-      <c r="K10" s="57"/>
+      <c r="B10" s="70"/>
+      <c r="C10" s="70"/>
+      <c r="D10" s="70"/>
+      <c r="E10" s="70"/>
+      <c r="F10" s="70"/>
+      <c r="G10" s="70"/>
+      <c r="H10" s="70"/>
+      <c r="I10" s="70"/>
+      <c r="J10" s="70"/>
+      <c r="K10" s="74"/>
       <c r="L10" s="35">
         <v>45889</v>
       </c>
@@ -1548,7 +1542,7 @@
         <v>15</v>
       </c>
       <c r="K11" s="23">
-        <v>0.75</v>
+        <v>0.9</v>
       </c>
       <c r="L11" s="37"/>
       <c r="M11" s="37"/>
@@ -1590,7 +1584,7 @@
         <v>45915</v>
       </c>
       <c r="H12" s="32" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="I12" s="32">
         <f t="shared" si="1"/>
@@ -1601,7 +1595,7 @@
         <v>8</v>
       </c>
       <c r="K12" s="23">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="L12" s="24"/>
       <c r="M12" s="25"/>
@@ -1642,8 +1636,8 @@
       <c r="G13" s="42">
         <v>45921</v>
       </c>
-      <c r="H13" s="53" t="s">
-        <v>60</v>
+      <c r="H13" s="71" t="s">
+        <v>59</v>
       </c>
       <c r="I13" s="32">
         <f t="shared" si="1"/>
@@ -1654,7 +1648,7 @@
         <v>7</v>
       </c>
       <c r="K13" s="23">
-        <v>0.1</v>
+        <v>0.7</v>
       </c>
       <c r="L13" s="24"/>
       <c r="M13" s="25"/>
@@ -1695,7 +1689,7 @@
       <c r="G14" s="42">
         <v>45919</v>
       </c>
-      <c r="H14" s="55"/>
+      <c r="H14" s="73"/>
       <c r="I14" s="32">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -1705,7 +1699,7 @@
         <v>5</v>
       </c>
       <c r="K14" s="23">
-        <v>0.1</v>
+        <v>0.5</v>
       </c>
       <c r="L14" s="24"/>
       <c r="M14" s="25"/>
@@ -1746,8 +1740,8 @@
       <c r="G15" s="42">
         <v>45919</v>
       </c>
-      <c r="H15" s="53" t="s">
-        <v>61</v>
+      <c r="H15" s="71" t="s">
+        <v>60</v>
       </c>
       <c r="I15" s="32">
         <f t="shared" ref="I15:I25" si="5">G15-F15</f>
@@ -1758,7 +1752,7 @@
         <v>5</v>
       </c>
       <c r="K15" s="23">
-        <v>0.1</v>
+        <v>0.9</v>
       </c>
       <c r="L15" s="24"/>
       <c r="M15" s="25"/>
@@ -1799,7 +1793,7 @@
       <c r="G16" s="42">
         <v>45919</v>
       </c>
-      <c r="H16" s="55"/>
+      <c r="H16" s="73"/>
       <c r="I16" s="32">
         <f t="shared" si="5"/>
         <v>0</v>
@@ -1809,7 +1803,7 @@
         <v>5</v>
       </c>
       <c r="K16" s="23">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="L16" s="24"/>
       <c r="M16" s="25"/>
@@ -1851,7 +1845,7 @@
         <v>45923</v>
       </c>
       <c r="H17" s="32" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I17" s="32">
         <f t="shared" si="5"/>
@@ -1862,7 +1856,7 @@
         <v>5</v>
       </c>
       <c r="K17" s="23">
-        <v>0.1</v>
+        <v>0.5</v>
       </c>
       <c r="L17" s="24"/>
       <c r="M17" s="25"/>
@@ -1904,7 +1898,7 @@
         <v>45923</v>
       </c>
       <c r="H18" s="32" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I18" s="32">
         <f t="shared" si="5"/>
@@ -1915,7 +1909,7 @@
         <v>5</v>
       </c>
       <c r="K18" s="23">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="L18" s="24"/>
       <c r="M18" s="25"/>
@@ -1941,32 +1935,31 @@
         <v>9</v>
       </c>
       <c r="C19" s="44" t="s">
-        <v>52</v>
+        <v>73</v>
       </c>
       <c r="D19" s="45" t="s">
         <v>36</v>
       </c>
       <c r="E19" s="46">
-        <f>G17</f>
-        <v>45923</v>
+        <v>45921</v>
       </c>
       <c r="F19" s="46">
-        <f t="shared" si="4"/>
-        <v>45930</v>
+        <f>G19</f>
+        <v>45928</v>
       </c>
       <c r="G19" s="46">
         <f>E19+7</f>
-        <v>45930</v>
+        <v>45928</v>
       </c>
       <c r="H19" s="32" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="I19" s="32">
-        <f t="shared" si="5"/>
+        <f>G19-F19</f>
         <v>0</v>
       </c>
       <c r="J19" s="32">
-        <f t="shared" si="6"/>
+        <f>DAYS360(E19,F19)+1</f>
         <v>8</v>
       </c>
       <c r="K19" s="23">
@@ -1996,32 +1989,31 @@
         <v>10</v>
       </c>
       <c r="C20" s="44" t="s">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="D20" s="45" t="s">
         <v>36</v>
       </c>
       <c r="E20" s="46">
-        <v>45921</v>
+        <v>45923</v>
       </c>
       <c r="F20" s="46">
-        <f t="shared" si="4"/>
-        <v>45928</v>
+        <f>G20</f>
+        <v>45943</v>
       </c>
       <c r="G20" s="46">
-        <f>E20+7</f>
-        <v>45928</v>
+        <v>45943</v>
       </c>
       <c r="H20" s="32" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I20" s="32">
-        <f t="shared" si="5"/>
+        <f>G20-F20</f>
         <v>0</v>
       </c>
       <c r="J20" s="32">
-        <f t="shared" si="6"/>
-        <v>8</v>
+        <f>DAYS360(E20,F20)+1</f>
+        <v>21</v>
       </c>
       <c r="K20" s="23">
         <v>0</v>
@@ -2050,31 +2042,31 @@
         <v>11</v>
       </c>
       <c r="C21" s="44" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D21" s="45" t="s">
         <v>36</v>
       </c>
       <c r="E21" s="46">
-        <v>45923</v>
+        <v>45925</v>
       </c>
       <c r="F21" s="46">
-        <f t="shared" si="4"/>
+        <f>G21</f>
         <v>45943</v>
       </c>
       <c r="G21" s="46">
         <v>45943</v>
       </c>
       <c r="H21" s="53" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="I21" s="32">
-        <f t="shared" si="5"/>
+        <f>G21-F21</f>
         <v>0</v>
       </c>
       <c r="J21" s="32">
-        <f t="shared" si="6"/>
-        <v>21</v>
+        <f>DAYS360(E21,F21)+1</f>
+        <v>19</v>
       </c>
       <c r="K21" s="23">
         <v>0</v>
@@ -2097,35 +2089,37 @@
       <c r="AA21" s="26"/>
       <c r="AB21" s="29"/>
     </row>
-    <row r="22" spans="1:28" ht="26.25" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:28" ht="61.5" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A22" s="22"/>
       <c r="B22" s="45">
         <v>12</v>
       </c>
       <c r="C22" s="44" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D22" s="45" t="s">
         <v>36</v>
       </c>
       <c r="E22" s="46">
-        <v>45925</v>
+        <v>45930</v>
       </c>
       <c r="F22" s="46">
-        <f t="shared" si="4"/>
-        <v>45943</v>
+        <f>G22</f>
+        <v>45931</v>
       </c>
       <c r="G22" s="46">
-        <v>45943</v>
-      </c>
-      <c r="H22" s="55"/>
+        <v>45931</v>
+      </c>
+      <c r="H22" s="32" t="s">
+        <v>66</v>
+      </c>
       <c r="I22" s="32">
-        <f t="shared" si="5"/>
+        <f>G22-F22</f>
         <v>0</v>
       </c>
       <c r="J22" s="32">
-        <f t="shared" si="6"/>
-        <v>19</v>
+        <f>DAYS360(E22,F22)+1</f>
+        <v>2</v>
       </c>
       <c r="K22" s="23">
         <v>0</v>
@@ -2154,31 +2148,31 @@
         <v>13</v>
       </c>
       <c r="C23" s="44" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D23" s="45" t="s">
         <v>36</v>
       </c>
       <c r="E23" s="46">
-        <v>45930</v>
+        <v>45931</v>
       </c>
       <c r="F23" s="46">
-        <f>G23</f>
-        <v>45931</v>
+        <f t="shared" ref="F23:F29" si="7">G23</f>
+        <v>45943</v>
       </c>
       <c r="G23" s="46">
-        <v>45931</v>
+        <v>45943</v>
       </c>
       <c r="H23" s="32" t="s">
         <v>67</v>
       </c>
       <c r="I23" s="32">
-        <f t="shared" si="5"/>
+        <f>G23-F23</f>
         <v>0</v>
       </c>
       <c r="J23" s="32">
-        <f t="shared" si="6"/>
-        <v>2</v>
+        <f>DAYS360(E23,F23)+1</f>
+        <v>13</v>
       </c>
       <c r="K23" s="23">
         <v>0</v>
@@ -2203,35 +2197,35 @@
     </row>
     <row r="24" spans="1:28" ht="26.25" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A24" s="22"/>
-      <c r="B24" s="45">
+      <c r="B24" s="48">
         <v>14</v>
       </c>
-      <c r="C24" s="44" t="s">
-        <v>46</v>
-      </c>
-      <c r="D24" s="45" t="s">
+      <c r="C24" s="47" t="s">
+        <v>47</v>
+      </c>
+      <c r="D24" s="48" t="s">
         <v>36</v>
       </c>
-      <c r="E24" s="46">
-        <v>45931</v>
-      </c>
-      <c r="F24" s="46">
-        <f t="shared" ref="F24:F30" si="7">G24</f>
+      <c r="E24" s="49">
         <v>45943</v>
       </c>
-      <c r="G24" s="46">
-        <v>45943</v>
-      </c>
-      <c r="H24" s="32" t="s">
+      <c r="F24" s="49">
+        <f t="shared" si="7"/>
+        <v>45961</v>
+      </c>
+      <c r="G24" s="49">
+        <v>45961</v>
+      </c>
+      <c r="H24" s="71" t="s">
         <v>68</v>
       </c>
       <c r="I24" s="32">
-        <f t="shared" si="5"/>
+        <f>G24-F24</f>
         <v>0</v>
       </c>
       <c r="J24" s="32">
-        <f t="shared" si="6"/>
-        <v>13</v>
+        <f>DAYS360(E24,F24)+1</f>
+        <v>19</v>
       </c>
       <c r="K24" s="23">
         <v>0</v>
@@ -2260,31 +2254,29 @@
         <v>15</v>
       </c>
       <c r="C25" s="47" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="D25" s="48" t="s">
         <v>36</v>
       </c>
       <c r="E25" s="49">
-        <v>45943</v>
+        <v>45962</v>
       </c>
       <c r="F25" s="49">
         <f t="shared" si="7"/>
-        <v>45961</v>
+        <v>45968</v>
       </c>
       <c r="G25" s="49">
-        <v>45961</v>
-      </c>
-      <c r="H25" s="53" t="s">
-        <v>69</v>
-      </c>
+        <v>45968</v>
+      </c>
+      <c r="H25" s="72"/>
       <c r="I25" s="32">
-        <f t="shared" si="5"/>
+        <f>G25-F25</f>
         <v>0</v>
       </c>
       <c r="J25" s="32">
-        <f t="shared" si="6"/>
-        <v>19</v>
+        <f>DAYS360(E25,F25)+1</f>
+        <v>7</v>
       </c>
       <c r="K25" s="23">
         <v>0</v>
@@ -2319,23 +2311,24 @@
         <v>36</v>
       </c>
       <c r="E26" s="49">
-        <v>45962</v>
+        <f>G25</f>
+        <v>45968</v>
       </c>
       <c r="F26" s="49">
         <f t="shared" si="7"/>
-        <v>45968</v>
+        <v>45975</v>
       </c>
       <c r="G26" s="49">
-        <v>45968</v>
-      </c>
-      <c r="H26" s="54"/>
+        <v>45975</v>
+      </c>
+      <c r="H26" s="73"/>
       <c r="I26" s="32">
-        <f t="shared" si="1"/>
+        <f>G26-F26</f>
         <v>0</v>
       </c>
       <c r="J26" s="32">
-        <f t="shared" si="2"/>
-        <v>7</v>
+        <f>DAYS360(E26,F26)+1</f>
+        <v>8</v>
       </c>
       <c r="K26" s="23">
         <v>0</v>
@@ -2360,34 +2353,36 @@
     </row>
     <row r="27" spans="1:28" ht="30.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A27" s="30"/>
-      <c r="B27" s="48">
+      <c r="B27" s="32">
         <v>17</v>
       </c>
-      <c r="C27" s="47" t="s">
+      <c r="C27" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="D27" s="48" t="s">
+      <c r="D27" s="32" t="s">
         <v>36</v>
       </c>
-      <c r="E27" s="49">
-        <f>G26</f>
-        <v>45968</v>
-      </c>
-      <c r="F27" s="49">
+      <c r="E27" s="34">
+        <f>E25</f>
+        <v>45962</v>
+      </c>
+      <c r="F27" s="34">
         <f t="shared" si="7"/>
-        <v>45975</v>
-      </c>
-      <c r="G27" s="49">
-        <v>45975</v>
-      </c>
-      <c r="H27" s="55"/>
+        <v>45991</v>
+      </c>
+      <c r="G27" s="34">
+        <v>45991</v>
+      </c>
+      <c r="H27" s="71" t="s">
+        <v>69</v>
+      </c>
       <c r="I27" s="32">
-        <f t="shared" si="1"/>
+        <f>G27-F27</f>
         <v>0</v>
       </c>
       <c r="J27" s="32">
-        <f t="shared" si="2"/>
-        <v>8</v>
+        <f>DAYS360(E27,F27)+1</f>
+        <v>30</v>
       </c>
       <c r="K27" s="23">
         <v>0</v>
@@ -2412,18 +2407,18 @@
     </row>
     <row r="28" spans="1:28" ht="30" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A28" s="22"/>
-      <c r="B28" s="74">
+      <c r="B28" s="32">
         <v>18</v>
       </c>
       <c r="C28" s="33" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="D28" s="32" t="s">
         <v>36</v>
       </c>
       <c r="E28" s="34">
-        <f>E26</f>
-        <v>45962</v>
+        <f>G26</f>
+        <v>45975</v>
       </c>
       <c r="F28" s="34">
         <f t="shared" si="7"/>
@@ -2432,16 +2427,14 @@
       <c r="G28" s="34">
         <v>45991</v>
       </c>
-      <c r="H28" s="53" t="s">
-        <v>70</v>
-      </c>
+      <c r="H28" s="72"/>
       <c r="I28" s="32">
-        <f t="shared" si="1"/>
+        <f>G28-F28</f>
         <v>0</v>
       </c>
       <c r="J28" s="32">
-        <f t="shared" si="2"/>
-        <v>30</v>
+        <f>DAYS360(E28,F28)+1</f>
+        <v>17</v>
       </c>
       <c r="K28" s="23">
         <v>0</v>
@@ -2466,17 +2459,16 @@
     </row>
     <row r="29" spans="1:28" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A29" s="22"/>
-      <c r="B29" s="75">
+      <c r="B29" s="32">
         <v>19</v>
       </c>
       <c r="C29" s="33" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D29" s="32" t="s">
         <v>36</v>
       </c>
       <c r="E29" s="34">
-        <f>G27</f>
         <v>45975</v>
       </c>
       <c r="F29" s="34">
@@ -2486,13 +2478,13 @@
       <c r="G29" s="34">
         <v>45991</v>
       </c>
-      <c r="H29" s="54"/>
+      <c r="H29" s="73"/>
       <c r="I29" s="32">
-        <f t="shared" si="1"/>
+        <f>G29-F29</f>
         <v>0</v>
       </c>
       <c r="J29" s="32">
-        <f t="shared" si="2"/>
+        <f>DAYS360(E29,F29)+1</f>
         <v>17</v>
       </c>
       <c r="K29" s="23">
@@ -2518,33 +2510,36 @@
     </row>
     <row r="30" spans="1:28" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A30" s="30"/>
-      <c r="B30" s="74">
+      <c r="B30" s="32">
         <v>20</v>
       </c>
       <c r="C30" s="33" t="s">
-        <v>54</v>
-      </c>
-      <c r="D30" s="32" t="s">
+        <v>52</v>
+      </c>
+      <c r="D30" s="33" t="s">
         <v>36</v>
       </c>
       <c r="E30" s="34">
         <v>45975</v>
       </c>
       <c r="F30" s="34">
-        <f t="shared" si="7"/>
-        <v>45991</v>
+        <f>G30</f>
+        <v>45982</v>
       </c>
       <c r="G30" s="34">
-        <v>45991</v>
-      </c>
-      <c r="H30" s="55"/>
+        <f>E30+7</f>
+        <v>45982</v>
+      </c>
+      <c r="H30" s="32" t="s">
+        <v>63</v>
+      </c>
       <c r="I30" s="32">
-        <f t="shared" si="1"/>
+        <f>G30-F30</f>
         <v>0</v>
       </c>
       <c r="J30" s="32">
-        <f t="shared" si="2"/>
-        <v>17</v>
+        <f>DAYS360(E30,F30)+1</f>
+        <v>8</v>
       </c>
       <c r="K30" s="23">
         <v>0</v>
@@ -2569,16 +2564,6 @@
     </row>
     <row r="31" spans="1:28" ht="17.25" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A31" s="30"/>
-      <c r="B31" s="36"/>
-      <c r="C31" s="36"/>
-      <c r="D31" s="36"/>
-      <c r="E31" s="36"/>
-      <c r="F31" s="36"/>
-      <c r="G31" s="36"/>
-      <c r="H31" s="36"/>
-      <c r="I31" s="36"/>
-      <c r="J31" s="36"/>
-      <c r="K31" s="36"/>
       <c r="L31" s="36"/>
       <c r="M31" s="36"/>
       <c r="N31" s="36"/>
@@ -2690,13 +2675,13 @@
     <row r="35" spans="1:28" ht="17.25" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A35" s="22"/>
       <c r="B35" s="40" t="s">
+        <v>70</v>
+      </c>
+      <c r="C35" s="45" t="s">
         <v>71</v>
       </c>
-      <c r="C35" s="45" t="s">
+      <c r="D35" s="48" t="s">
         <v>72</v>
-      </c>
-      <c r="D35" s="48" t="s">
-        <v>73</v>
       </c>
       <c r="E35" s="36"/>
       <c r="F35" s="36"/>
@@ -3704,21 +3689,12 @@
     <row r="957" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="958" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
-  <mergeCells count="31">
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="L4:X4"/>
-    <mergeCell ref="D6:O6"/>
-    <mergeCell ref="D4:H4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="D5:H5"/>
-    <mergeCell ref="J5:K5"/>
-    <mergeCell ref="B2:K2"/>
-    <mergeCell ref="L2:AA2"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="D3:K3"/>
-    <mergeCell ref="L3:T3"/>
-    <mergeCell ref="U3:AA3"/>
+  <mergeCells count="30">
+    <mergeCell ref="K8:K10"/>
+    <mergeCell ref="H13:H14"/>
+    <mergeCell ref="H15:H16"/>
+    <mergeCell ref="H27:H29"/>
+    <mergeCell ref="H24:H26"/>
     <mergeCell ref="B8:B10"/>
     <mergeCell ref="C8:C10"/>
     <mergeCell ref="D8:D10"/>
@@ -3730,12 +3706,20 @@
     <mergeCell ref="H8:H10"/>
     <mergeCell ref="I8:I10"/>
     <mergeCell ref="J8:J10"/>
-    <mergeCell ref="H28:H30"/>
-    <mergeCell ref="K8:K10"/>
-    <mergeCell ref="H13:H14"/>
-    <mergeCell ref="H15:H16"/>
-    <mergeCell ref="H21:H22"/>
-    <mergeCell ref="H25:H27"/>
+    <mergeCell ref="B2:K2"/>
+    <mergeCell ref="L2:AA2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="D3:K3"/>
+    <mergeCell ref="L3:T3"/>
+    <mergeCell ref="U3:AA3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="L4:X4"/>
+    <mergeCell ref="D6:O6"/>
+    <mergeCell ref="D4:H4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="D5:H5"/>
+    <mergeCell ref="J5:K5"/>
   </mergeCells>
   <phoneticPr fontId="23" type="noConversion"/>
   <conditionalFormatting sqref="L10:AA10">

</xml_diff>

<commit_message>
Avance-1: - Documento de Avance-1 - Reporte de Avance-1
</commit_message>
<xml_diff>
--- a/REPORTES/Cronograma-MHinojosa.xlsx
+++ b/REPORTES/Cronograma-MHinojosa.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Desktop\TESIS 2\TFC2_20212123_MHinojosa\TFC2-20212123-LaTeX\REPORTES\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12EC6E21-AA59-4D5F-92FF-18F556C4B791}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86C60CE0-7DF3-43BC-BDEC-6C61DED87F99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11310" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -747,20 +747,64 @@
     <xf numFmtId="0" fontId="19" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="19" fillId="10" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="14" fontId="19" fillId="11" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="19" fillId="11" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="19" fillId="10" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="20" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -781,61 +825,17 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="19" fillId="10" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="19" fillId="11" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="19" fillId="11" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="19" fillId="10" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="20" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1078,7 +1078,7 @@
     <col min="3" max="3" width="26.85546875" customWidth="1"/>
     <col min="4" max="4" width="13.5703125" customWidth="1"/>
     <col min="5" max="7" width="11" customWidth="1"/>
-    <col min="8" max="8" width="42.5703125" style="71" customWidth="1"/>
+    <col min="8" max="8" width="42.5703125" style="53" customWidth="1"/>
     <col min="9" max="9" width="10.85546875" customWidth="1"/>
     <col min="10" max="10" width="12.42578125" customWidth="1"/>
     <col min="11" max="11" width="14.85546875" customWidth="1"/>
@@ -1096,7 +1096,7 @@
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
-      <c r="H1" s="70"/>
+      <c r="H1" s="52"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
@@ -1119,131 +1119,131 @@
     </row>
     <row r="2" spans="1:28" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
-      <c r="B2" s="48" t="s">
+      <c r="B2" s="66" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="49"/>
-      <c r="D2" s="49"/>
-      <c r="E2" s="49"/>
-      <c r="F2" s="49"/>
-      <c r="G2" s="49"/>
-      <c r="H2" s="49"/>
-      <c r="I2" s="49"/>
-      <c r="J2" s="49"/>
-      <c r="K2" s="49"/>
-      <c r="L2" s="50"/>
-      <c r="M2" s="49"/>
-      <c r="N2" s="49"/>
-      <c r="O2" s="49"/>
-      <c r="P2" s="49"/>
-      <c r="Q2" s="49"/>
-      <c r="R2" s="49"/>
-      <c r="S2" s="49"/>
-      <c r="T2" s="49"/>
-      <c r="U2" s="49"/>
-      <c r="V2" s="49"/>
-      <c r="W2" s="49"/>
-      <c r="X2" s="49"/>
-      <c r="Y2" s="49"/>
-      <c r="Z2" s="49"/>
-      <c r="AA2" s="49"/>
+      <c r="C2" s="67"/>
+      <c r="D2" s="67"/>
+      <c r="E2" s="67"/>
+      <c r="F2" s="67"/>
+      <c r="G2" s="67"/>
+      <c r="H2" s="67"/>
+      <c r="I2" s="67"/>
+      <c r="J2" s="67"/>
+      <c r="K2" s="67"/>
+      <c r="L2" s="68"/>
+      <c r="M2" s="67"/>
+      <c r="N2" s="67"/>
+      <c r="O2" s="67"/>
+      <c r="P2" s="67"/>
+      <c r="Q2" s="67"/>
+      <c r="R2" s="67"/>
+      <c r="S2" s="67"/>
+      <c r="T2" s="67"/>
+      <c r="U2" s="67"/>
+      <c r="V2" s="67"/>
+      <c r="W2" s="67"/>
+      <c r="X2" s="67"/>
+      <c r="Y2" s="67"/>
+      <c r="Z2" s="67"/>
+      <c r="AA2" s="67"/>
     </row>
     <row r="3" spans="1:28" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A3" s="3"/>
-      <c r="B3" s="51"/>
-      <c r="C3" s="52"/>
-      <c r="D3" s="53"/>
-      <c r="E3" s="52"/>
-      <c r="F3" s="52"/>
-      <c r="G3" s="52"/>
-      <c r="H3" s="52"/>
-      <c r="I3" s="52"/>
-      <c r="J3" s="52"/>
-      <c r="K3" s="52"/>
-      <c r="L3" s="54"/>
-      <c r="M3" s="52"/>
-      <c r="N3" s="52"/>
-      <c r="O3" s="52"/>
-      <c r="P3" s="52"/>
-      <c r="Q3" s="52"/>
-      <c r="R3" s="52"/>
-      <c r="S3" s="52"/>
-      <c r="T3" s="52"/>
-      <c r="U3" s="55"/>
-      <c r="V3" s="52"/>
-      <c r="W3" s="52"/>
-      <c r="X3" s="52"/>
-      <c r="Y3" s="52"/>
-      <c r="Z3" s="52"/>
-      <c r="AA3" s="52"/>
+      <c r="B3" s="69"/>
+      <c r="C3" s="70"/>
+      <c r="D3" s="71"/>
+      <c r="E3" s="70"/>
+      <c r="F3" s="70"/>
+      <c r="G3" s="70"/>
+      <c r="H3" s="70"/>
+      <c r="I3" s="70"/>
+      <c r="J3" s="70"/>
+      <c r="K3" s="70"/>
+      <c r="L3" s="72"/>
+      <c r="M3" s="70"/>
+      <c r="N3" s="70"/>
+      <c r="O3" s="70"/>
+      <c r="P3" s="70"/>
+      <c r="Q3" s="70"/>
+      <c r="R3" s="70"/>
+      <c r="S3" s="70"/>
+      <c r="T3" s="70"/>
+      <c r="U3" s="73"/>
+      <c r="V3" s="70"/>
+      <c r="W3" s="70"/>
+      <c r="X3" s="70"/>
+      <c r="Y3" s="70"/>
+      <c r="Z3" s="70"/>
+      <c r="AA3" s="70"/>
     </row>
     <row r="4" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="4"/>
-      <c r="B4" s="47" t="s">
+      <c r="B4" s="59" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="46"/>
-      <c r="D4" s="57" t="s">
+      <c r="C4" s="60"/>
+      <c r="D4" s="63" t="s">
         <v>20</v>
       </c>
-      <c r="E4" s="46"/>
-      <c r="F4" s="46"/>
-      <c r="G4" s="46"/>
-      <c r="H4" s="46"/>
+      <c r="E4" s="60"/>
+      <c r="F4" s="60"/>
+      <c r="G4" s="60"/>
+      <c r="H4" s="60"/>
       <c r="I4" s="5"/>
-      <c r="J4" s="47" t="s">
+      <c r="J4" s="59" t="s">
         <v>2</v>
       </c>
-      <c r="K4" s="46"/>
-      <c r="L4" s="56"/>
-      <c r="M4" s="46"/>
-      <c r="N4" s="46"/>
-      <c r="O4" s="46"/>
-      <c r="P4" s="46"/>
-      <c r="Q4" s="46"/>
-      <c r="R4" s="46"/>
-      <c r="S4" s="46"/>
-      <c r="T4" s="46"/>
-      <c r="U4" s="46"/>
-      <c r="V4" s="46"/>
-      <c r="W4" s="46"/>
-      <c r="X4" s="46"/>
+      <c r="K4" s="60"/>
+      <c r="L4" s="61"/>
+      <c r="M4" s="60"/>
+      <c r="N4" s="60"/>
+      <c r="O4" s="60"/>
+      <c r="P4" s="60"/>
+      <c r="Q4" s="60"/>
+      <c r="R4" s="60"/>
+      <c r="S4" s="60"/>
+      <c r="T4" s="60"/>
+      <c r="U4" s="60"/>
+      <c r="V4" s="60"/>
+      <c r="W4" s="60"/>
+      <c r="X4" s="60"/>
       <c r="Y4" s="6"/>
       <c r="Z4" s="6"/>
       <c r="AA4" s="6"/>
     </row>
     <row r="5" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="4"/>
-      <c r="B5" s="47" t="s">
+      <c r="B5" s="59" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="46"/>
-      <c r="D5" s="58" t="s">
+      <c r="C5" s="60"/>
+      <c r="D5" s="64" t="s">
         <v>21</v>
       </c>
-      <c r="E5" s="46"/>
-      <c r="F5" s="46"/>
-      <c r="G5" s="46"/>
-      <c r="H5" s="46"/>
+      <c r="E5" s="60"/>
+      <c r="F5" s="60"/>
+      <c r="G5" s="60"/>
+      <c r="H5" s="60"/>
       <c r="I5" s="8"/>
-      <c r="J5" s="59" t="s">
+      <c r="J5" s="65" t="s">
         <v>24</v>
       </c>
-      <c r="K5" s="46"/>
-      <c r="L5" s="45">
+      <c r="K5" s="60"/>
+      <c r="L5" s="62">
         <v>46081</v>
       </c>
-      <c r="M5" s="46"/>
-      <c r="N5" s="46"/>
-      <c r="O5" s="46"/>
-      <c r="P5" s="46"/>
-      <c r="Q5" s="46"/>
-      <c r="R5" s="46"/>
-      <c r="S5" s="46"/>
-      <c r="T5" s="46"/>
-      <c r="U5" s="46"/>
-      <c r="V5" s="46"/>
-      <c r="W5" s="46"/>
+      <c r="M5" s="60"/>
+      <c r="N5" s="60"/>
+      <c r="O5" s="60"/>
+      <c r="P5" s="60"/>
+      <c r="Q5" s="60"/>
+      <c r="R5" s="60"/>
+      <c r="S5" s="60"/>
+      <c r="T5" s="60"/>
+      <c r="U5" s="60"/>
+      <c r="V5" s="60"/>
+      <c r="W5" s="60"/>
       <c r="X5" s="9"/>
       <c r="Y5" s="9"/>
       <c r="Z5" s="9"/>
@@ -1251,25 +1251,25 @@
     </row>
     <row r="6" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="4"/>
-      <c r="B6" s="47" t="s">
+      <c r="B6" s="59" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="46"/>
-      <c r="D6" s="45">
+      <c r="C6" s="60"/>
+      <c r="D6" s="62">
         <f>L5-54</f>
         <v>46027</v>
       </c>
-      <c r="E6" s="46"/>
-      <c r="F6" s="46"/>
-      <c r="G6" s="46"/>
-      <c r="H6" s="46"/>
-      <c r="I6" s="46"/>
-      <c r="J6" s="46"/>
-      <c r="K6" s="46"/>
-      <c r="L6" s="46"/>
-      <c r="M6" s="46"/>
-      <c r="N6" s="46"/>
-      <c r="O6" s="46"/>
+      <c r="E6" s="60"/>
+      <c r="F6" s="60"/>
+      <c r="G6" s="60"/>
+      <c r="H6" s="60"/>
+      <c r="I6" s="60"/>
+      <c r="J6" s="60"/>
+      <c r="K6" s="60"/>
+      <c r="L6" s="60"/>
+      <c r="M6" s="60"/>
+      <c r="N6" s="60"/>
+      <c r="O6" s="60"/>
       <c r="P6" s="8"/>
       <c r="Q6" s="8"/>
       <c r="R6" s="8"/>
@@ -1292,7 +1292,7 @@
       <c r="E7" s="13"/>
       <c r="F7" s="13"/>
       <c r="G7" s="13"/>
-      <c r="H7" s="72"/>
+      <c r="H7" s="54"/>
       <c r="I7" s="13"/>
       <c r="J7" s="13"/>
       <c r="K7" s="13"/>
@@ -1316,34 +1316,34 @@
     </row>
     <row r="8" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="14"/>
-      <c r="B8" s="42" t="s">
+      <c r="B8" s="74" t="s">
         <v>48</v>
       </c>
-      <c r="C8" s="42" t="s">
+      <c r="C8" s="74" t="s">
         <v>8</v>
       </c>
-      <c r="D8" s="42" t="s">
+      <c r="D8" s="74" t="s">
         <v>9</v>
       </c>
-      <c r="E8" s="42" t="s">
+      <c r="E8" s="74" t="s">
         <v>10</v>
       </c>
-      <c r="F8" s="42" t="s">
+      <c r="F8" s="74" t="s">
         <v>11</v>
       </c>
-      <c r="G8" s="42" t="s">
+      <c r="G8" s="74" t="s">
         <v>12</v>
       </c>
-      <c r="H8" s="73" t="s">
+      <c r="H8" s="76" t="s">
         <v>13</v>
       </c>
-      <c r="I8" s="42" t="s">
+      <c r="I8" s="74" t="s">
         <v>14</v>
       </c>
-      <c r="J8" s="42" t="s">
+      <c r="J8" s="74" t="s">
         <v>15</v>
       </c>
-      <c r="K8" s="42" t="s">
+      <c r="K8" s="74" t="s">
         <v>16</v>
       </c>
       <c r="L8" s="15"/>
@@ -1366,16 +1366,16 @@
     </row>
     <row r="9" spans="1:28" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="16"/>
-      <c r="B9" s="42"/>
-      <c r="C9" s="42"/>
-      <c r="D9" s="42"/>
-      <c r="E9" s="42"/>
-      <c r="F9" s="42"/>
-      <c r="G9" s="42"/>
-      <c r="H9" s="73"/>
-      <c r="I9" s="42"/>
-      <c r="J9" s="42"/>
-      <c r="K9" s="42"/>
+      <c r="B9" s="74"/>
+      <c r="C9" s="74"/>
+      <c r="D9" s="74"/>
+      <c r="E9" s="74"/>
+      <c r="F9" s="74"/>
+      <c r="G9" s="74"/>
+      <c r="H9" s="76"/>
+      <c r="I9" s="74"/>
+      <c r="J9" s="74"/>
+      <c r="K9" s="74"/>
       <c r="L9" s="17" t="s">
         <v>5</v>
       </c>
@@ -1428,16 +1428,16 @@
     </row>
     <row r="10" spans="1:28" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="19"/>
-      <c r="B10" s="44"/>
-      <c r="C10" s="44"/>
-      <c r="D10" s="44"/>
-      <c r="E10" s="44"/>
-      <c r="F10" s="44"/>
-      <c r="G10" s="44"/>
-      <c r="H10" s="73"/>
-      <c r="I10" s="44"/>
-      <c r="J10" s="44"/>
-      <c r="K10" s="43"/>
+      <c r="B10" s="75"/>
+      <c r="C10" s="75"/>
+      <c r="D10" s="75"/>
+      <c r="E10" s="75"/>
+      <c r="F10" s="75"/>
+      <c r="G10" s="75"/>
+      <c r="H10" s="76"/>
+      <c r="I10" s="75"/>
+      <c r="J10" s="75"/>
+      <c r="K10" s="77"/>
       <c r="L10" s="32">
         <v>45889</v>
       </c>
@@ -1507,33 +1507,32 @@
       <c r="B11" s="35">
         <v>1</v>
       </c>
-      <c r="C11" s="64" t="s">
+      <c r="C11" s="46" t="s">
         <v>40</v>
       </c>
-      <c r="D11" s="65" t="s">
+      <c r="D11" s="47" t="s">
         <v>22</v>
       </c>
-      <c r="E11" s="66">
+      <c r="E11" s="48">
         <v>46027</v>
       </c>
-      <c r="F11" s="66">
-        <f>G11</f>
-        <v>46031</v>
-      </c>
-      <c r="G11" s="67">
+      <c r="F11" s="48">
+        <v>46034</v>
+      </c>
+      <c r="G11" s="49">
         <f>E11+4</f>
         <v>46031</v>
       </c>
       <c r="H11" s="41" t="s">
         <v>43</v>
       </c>
-      <c r="I11" s="69">
+      <c r="I11" s="51">
         <f t="shared" ref="I11:I14" si="1">G11-F11</f>
-        <v>0</v>
+        <v>-3</v>
       </c>
       <c r="J11" s="31">
         <f t="shared" ref="J11:J14" si="2">DAYS360(E11,F11)+1</f>
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="K11" s="22">
         <v>0.7</v>
@@ -1561,35 +1560,34 @@
       <c r="B12" s="36">
         <v>2</v>
       </c>
-      <c r="C12" s="64" t="s">
+      <c r="C12" s="46" t="s">
         <v>25</v>
       </c>
-      <c r="D12" s="65" t="s">
+      <c r="D12" s="47" t="s">
         <v>22</v>
       </c>
-      <c r="E12" s="66">
+      <c r="E12" s="48">
         <v>46027</v>
       </c>
-      <c r="F12" s="66">
-        <f>G12</f>
-        <v>46031</v>
-      </c>
-      <c r="G12" s="67">
+      <c r="F12" s="48">
+        <v>46034</v>
+      </c>
+      <c r="G12" s="49">
         <v>46031</v>
       </c>
       <c r="H12" s="31" t="s">
         <v>60</v>
       </c>
-      <c r="I12" s="69">
+      <c r="I12" s="51">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-3</v>
       </c>
       <c r="J12" s="31">
         <f t="shared" si="2"/>
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="K12" s="22">
-        <v>0.1</v>
+        <v>0.8</v>
       </c>
       <c r="L12" s="23"/>
       <c r="M12" s="24"/>
@@ -1614,33 +1612,32 @@
       <c r="B13" s="35">
         <v>3</v>
       </c>
-      <c r="C13" s="64" t="s">
+      <c r="C13" s="46" t="s">
         <v>42</v>
       </c>
-      <c r="D13" s="65" t="s">
+      <c r="D13" s="47" t="s">
         <v>22</v>
       </c>
-      <c r="E13" s="66">
+      <c r="E13" s="48">
         <v>46031</v>
       </c>
-      <c r="F13" s="66">
-        <f t="shared" ref="F13" si="3">G13</f>
-        <v>46031</v>
-      </c>
-      <c r="G13" s="67">
+      <c r="F13" s="48">
+        <v>46034</v>
+      </c>
+      <c r="G13" s="49">
         <f>G12</f>
         <v>46031</v>
       </c>
       <c r="H13" s="31" t="s">
         <v>44</v>
       </c>
-      <c r="I13" s="69">
+      <c r="I13" s="51">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-3</v>
       </c>
       <c r="J13" s="31">
         <f t="shared" si="2"/>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K13" s="22">
         <v>0.8</v>
@@ -1668,26 +1665,26 @@
       <c r="B14" s="35">
         <v>4</v>
       </c>
-      <c r="C14" s="64" t="s">
+      <c r="C14" s="46" t="s">
         <v>41</v>
       </c>
-      <c r="D14" s="65" t="s">
+      <c r="D14" s="47" t="s">
         <v>22</v>
       </c>
-      <c r="E14" s="66">
+      <c r="E14" s="48">
         <v>46031</v>
       </c>
-      <c r="F14" s="66">
+      <c r="F14" s="48">
         <f>G14</f>
         <v>46034</v>
       </c>
-      <c r="G14" s="67">
+      <c r="G14" s="49">
         <v>46034</v>
       </c>
       <c r="H14" s="31" t="s">
         <v>45</v>
       </c>
-      <c r="I14" s="69">
+      <c r="I14" s="51">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -1721,27 +1718,27 @@
       <c r="B15" s="35">
         <v>5</v>
       </c>
-      <c r="C15" s="60" t="s">
+      <c r="C15" s="42" t="s">
         <v>46</v>
       </c>
-      <c r="D15" s="61" t="s">
+      <c r="D15" s="43" t="s">
         <v>22</v>
       </c>
-      <c r="E15" s="62">
+      <c r="E15" s="44">
         <v>46034</v>
       </c>
-      <c r="F15" s="62">
+      <c r="F15" s="44">
         <f>G15</f>
         <v>46041</v>
       </c>
-      <c r="G15" s="68">
+      <c r="G15" s="50">
         <f>E15+7</f>
         <v>46041</v>
       </c>
       <c r="H15" s="31" t="s">
         <v>49</v>
       </c>
-      <c r="I15" s="69">
+      <c r="I15" s="51">
         <f>G15-F15</f>
         <v>0</v>
       </c>
@@ -1757,7 +1754,7 @@
       <c r="N15" s="24"/>
       <c r="O15" s="25"/>
       <c r="P15" s="37"/>
-      <c r="Q15" s="77"/>
+      <c r="Q15" s="58"/>
       <c r="R15" s="25"/>
       <c r="S15" s="25"/>
       <c r="T15" s="25"/>
@@ -1775,27 +1772,27 @@
       <c r="B16" s="36">
         <v>6</v>
       </c>
-      <c r="C16" s="60" t="s">
+      <c r="C16" s="42" t="s">
         <v>47</v>
       </c>
-      <c r="D16" s="61" t="s">
+      <c r="D16" s="43" t="s">
         <v>22</v>
       </c>
-      <c r="E16" s="62">
+      <c r="E16" s="44">
         <v>46037</v>
       </c>
-      <c r="F16" s="62">
+      <c r="F16" s="44">
         <f>G16</f>
         <v>46041</v>
       </c>
-      <c r="G16" s="68">
+      <c r="G16" s="50">
         <f>E16+4</f>
         <v>46041</v>
       </c>
       <c r="H16" s="31" t="s">
         <v>50</v>
       </c>
-      <c r="I16" s="69">
+      <c r="I16" s="51">
         <f>G16-F16</f>
         <v>0</v>
       </c>
@@ -1829,32 +1826,32 @@
       <c r="B17" s="35">
         <v>7</v>
       </c>
-      <c r="C17" s="60" t="s">
+      <c r="C17" s="42" t="s">
         <v>23</v>
       </c>
-      <c r="D17" s="61" t="s">
+      <c r="D17" s="43" t="s">
         <v>22</v>
       </c>
-      <c r="E17" s="62">
+      <c r="E17" s="44">
         <v>46041</v>
       </c>
-      <c r="F17" s="62">
+      <c r="F17" s="44">
         <f>G17</f>
         <v>46055</v>
       </c>
-      <c r="G17" s="68">
+      <c r="G17" s="50">
         <f>E17+14</f>
         <v>46055</v>
       </c>
       <c r="H17" s="31" t="s">
         <v>62</v>
       </c>
-      <c r="I17" s="69">
-        <f t="shared" ref="I17:I26" si="4">G17-F17</f>
+      <c r="I17" s="51">
+        <f t="shared" ref="I17:I26" si="3">G17-F17</f>
         <v>0</v>
       </c>
       <c r="J17" s="31">
-        <f t="shared" ref="J17:J26" si="5">DAYS360(E17,F17)+1</f>
+        <f t="shared" ref="J17:J20" si="4">DAYS360(E17,F17)+1</f>
         <v>14</v>
       </c>
       <c r="K17" s="22">
@@ -1867,7 +1864,7 @@
       <c r="P17" s="25"/>
       <c r="Q17" s="37"/>
       <c r="R17" s="37"/>
-      <c r="S17" s="77"/>
+      <c r="S17" s="58"/>
       <c r="T17" s="25"/>
       <c r="U17" s="25"/>
       <c r="V17" s="25"/>
@@ -1883,33 +1880,33 @@
       <c r="B18" s="35">
         <v>8</v>
       </c>
-      <c r="C18" s="60" t="s">
+      <c r="C18" s="42" t="s">
         <v>61</v>
       </c>
-      <c r="D18" s="61" t="s">
+      <c r="D18" s="43" t="s">
         <v>22</v>
       </c>
-      <c r="E18" s="62">
+      <c r="E18" s="44">
         <f>E17+7</f>
         <v>46048</v>
       </c>
-      <c r="F18" s="62">
+      <c r="F18" s="44">
         <f>G17</f>
         <v>46055</v>
       </c>
-      <c r="G18" s="68">
+      <c r="G18" s="50">
         <f>G17</f>
         <v>46055</v>
       </c>
       <c r="H18" s="31" t="s">
         <v>63</v>
       </c>
-      <c r="I18" s="69">
+      <c r="I18" s="51">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="J18" s="31">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="J18" s="31">
-        <f t="shared" si="5"/>
         <v>7</v>
       </c>
       <c r="K18" s="22">
@@ -1922,7 +1919,7 @@
       <c r="P18" s="25"/>
       <c r="Q18" s="25"/>
       <c r="R18" s="37"/>
-      <c r="S18" s="77"/>
+      <c r="S18" s="58"/>
       <c r="T18" s="25"/>
       <c r="U18" s="25"/>
       <c r="V18" s="25"/>
@@ -1938,32 +1935,32 @@
       <c r="B19" s="35">
         <v>9</v>
       </c>
-      <c r="C19" s="60" t="s">
+      <c r="C19" s="42" t="s">
         <v>51</v>
       </c>
-      <c r="D19" s="61" t="s">
+      <c r="D19" s="43" t="s">
         <v>22</v>
       </c>
-      <c r="E19" s="62">
+      <c r="E19" s="44">
         <v>46048</v>
       </c>
-      <c r="F19" s="62">
-        <f>G19</f>
+      <c r="F19" s="44">
+        <f t="shared" ref="F19:F26" si="5">G19</f>
         <v>46062</v>
       </c>
-      <c r="G19" s="68">
+      <c r="G19" s="50">
         <f>E19+14</f>
         <v>46062</v>
       </c>
       <c r="H19" s="31" t="s">
         <v>64</v>
       </c>
-      <c r="I19" s="69">
+      <c r="I19" s="51">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="J19" s="31">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="J19" s="31">
-        <f t="shared" si="5"/>
         <v>14</v>
       </c>
       <c r="K19" s="22">
@@ -1977,7 +1974,7 @@
       <c r="Q19" s="25"/>
       <c r="R19" s="37"/>
       <c r="S19" s="37"/>
-      <c r="T19" s="77"/>
+      <c r="T19" s="58"/>
       <c r="U19" s="25"/>
       <c r="V19" s="25"/>
       <c r="W19" s="25"/>
@@ -1992,32 +1989,32 @@
       <c r="B20" s="36">
         <v>10</v>
       </c>
-      <c r="C20" s="60" t="s">
+      <c r="C20" s="42" t="s">
         <v>52</v>
       </c>
-      <c r="D20" s="61" t="s">
+      <c r="D20" s="43" t="s">
         <v>22</v>
       </c>
-      <c r="E20" s="62">
+      <c r="E20" s="44">
         <v>46041</v>
       </c>
-      <c r="F20" s="62">
-        <f>G20</f>
+      <c r="F20" s="44">
+        <f t="shared" si="5"/>
         <v>46044</v>
       </c>
-      <c r="G20" s="68">
+      <c r="G20" s="50">
         <f>E20+3</f>
         <v>46044</v>
       </c>
       <c r="H20" s="31" t="s">
         <v>65</v>
       </c>
-      <c r="I20" s="69">
+      <c r="I20" s="51">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="J20" s="31">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="J20" s="31">
-        <f t="shared" si="5"/>
         <v>4</v>
       </c>
       <c r="K20" s="22">
@@ -2046,32 +2043,32 @@
       <c r="B21" s="35">
         <v>11</v>
       </c>
-      <c r="C21" s="60" t="s">
+      <c r="C21" s="42" t="s">
         <v>53</v>
       </c>
-      <c r="D21" s="61" t="s">
+      <c r="D21" s="43" t="s">
         <v>22</v>
       </c>
-      <c r="E21" s="62">
+      <c r="E21" s="44">
         <v>46055</v>
       </c>
-      <c r="F21" s="62">
-        <f>G21</f>
+      <c r="F21" s="44">
+        <f t="shared" si="5"/>
         <v>46069</v>
       </c>
-      <c r="G21" s="68">
+      <c r="G21" s="50">
         <f>E21+14</f>
         <v>46069</v>
       </c>
       <c r="H21" s="31" t="s">
         <v>66</v>
       </c>
-      <c r="I21" s="69">
-        <f t="shared" si="4"/>
+      <c r="I21" s="51">
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J21" s="31">
-        <f t="shared" ref="J21:J26" si="6">G21-E21</f>
+        <f t="shared" ref="J21:J22" si="6">G21-E21</f>
         <v>14</v>
       </c>
       <c r="K21" s="22">
@@ -2086,7 +2083,7 @@
       <c r="R21" s="25"/>
       <c r="S21" s="37"/>
       <c r="T21" s="37"/>
-      <c r="U21" s="77"/>
+      <c r="U21" s="58"/>
       <c r="V21" s="25"/>
       <c r="W21" s="25"/>
       <c r="X21" s="25"/>
@@ -2100,28 +2097,28 @@
       <c r="B22" s="35">
         <v>12</v>
       </c>
-      <c r="C22" s="60" t="s">
+      <c r="C22" s="42" t="s">
         <v>54</v>
       </c>
-      <c r="D22" s="61" t="s">
+      <c r="D22" s="43" t="s">
         <v>22</v>
       </c>
-      <c r="E22" s="62">
+      <c r="E22" s="44">
         <v>46062</v>
       </c>
-      <c r="F22" s="62">
-        <f>G22</f>
+      <c r="F22" s="44">
+        <f t="shared" si="5"/>
         <v>46069</v>
       </c>
-      <c r="G22" s="68">
+      <c r="G22" s="50">
         <f>E22+7</f>
         <v>46069</v>
       </c>
-      <c r="H22" s="63" t="s">
+      <c r="H22" s="45" t="s">
         <v>69</v>
       </c>
-      <c r="I22" s="69">
-        <f t="shared" si="4"/>
+      <c r="I22" s="51">
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J22" s="31">
@@ -2140,7 +2137,7 @@
       <c r="R22" s="25"/>
       <c r="S22" s="25"/>
       <c r="T22" s="37"/>
-      <c r="U22" s="77"/>
+      <c r="U22" s="58"/>
       <c r="V22" s="25"/>
       <c r="W22" s="25"/>
       <c r="X22" s="25"/>
@@ -2154,28 +2151,28 @@
       <c r="B23" s="35">
         <v>13</v>
       </c>
-      <c r="C23" s="60" t="s">
+      <c r="C23" s="42" t="s">
         <v>55</v>
       </c>
-      <c r="D23" s="61" t="s">
+      <c r="D23" s="43" t="s">
         <v>22</v>
       </c>
-      <c r="E23" s="62">
+      <c r="E23" s="44">
         <v>46063</v>
       </c>
-      <c r="F23" s="62">
-        <f>G23</f>
+      <c r="F23" s="44">
+        <f t="shared" si="5"/>
         <v>46070</v>
       </c>
-      <c r="G23" s="68">
+      <c r="G23" s="50">
         <f>E23+7</f>
         <v>46070</v>
       </c>
-      <c r="H23" s="63" t="s">
+      <c r="H23" s="45" t="s">
         <v>67</v>
       </c>
-      <c r="I23" s="69">
-        <f t="shared" si="4"/>
+      <c r="I23" s="51">
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J23" s="31">
@@ -2208,28 +2205,28 @@
       <c r="B24" s="36">
         <v>14</v>
       </c>
-      <c r="C24" s="60" t="s">
+      <c r="C24" s="42" t="s">
         <v>56</v>
       </c>
-      <c r="D24" s="61" t="s">
+      <c r="D24" s="43" t="s">
         <v>22</v>
       </c>
-      <c r="E24" s="62">
+      <c r="E24" s="44">
         <v>46069</v>
       </c>
-      <c r="F24" s="62">
-        <f>G24</f>
+      <c r="F24" s="44">
+        <f t="shared" si="5"/>
         <v>46076</v>
       </c>
-      <c r="G24" s="68">
+      <c r="G24" s="50">
         <f>E24+7</f>
         <v>46076</v>
       </c>
-      <c r="H24" s="63" t="s">
+      <c r="H24" s="45" t="s">
         <v>68</v>
       </c>
-      <c r="I24" s="69">
-        <f t="shared" si="4"/>
+      <c r="I24" s="51">
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J24" s="31">
@@ -2262,28 +2259,28 @@
       <c r="B25" s="35">
         <v>15</v>
       </c>
-      <c r="C25" s="60" t="s">
+      <c r="C25" s="42" t="s">
         <v>26</v>
       </c>
-      <c r="D25" s="61" t="s">
+      <c r="D25" s="43" t="s">
         <v>22</v>
       </c>
-      <c r="E25" s="62">
+      <c r="E25" s="44">
         <v>46069</v>
       </c>
-      <c r="F25" s="62">
-        <f>G25</f>
+      <c r="F25" s="44">
+        <f t="shared" si="5"/>
         <v>46083</v>
       </c>
-      <c r="G25" s="68">
+      <c r="G25" s="50">
         <f>E25+14</f>
         <v>46083</v>
       </c>
       <c r="H25" s="31" t="s">
         <v>57</v>
       </c>
-      <c r="I25" s="69">
-        <f t="shared" si="4"/>
+      <c r="I25" s="51">
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J25" s="31">
@@ -2316,28 +2313,28 @@
       <c r="B26" s="35">
         <v>16</v>
       </c>
-      <c r="C26" s="60" t="s">
+      <c r="C26" s="42" t="s">
         <v>58</v>
       </c>
-      <c r="D26" s="60" t="s">
+      <c r="D26" s="42" t="s">
         <v>22</v>
       </c>
-      <c r="E26" s="62">
+      <c r="E26" s="44">
         <v>46069</v>
       </c>
-      <c r="F26" s="62">
-        <f>G26</f>
+      <c r="F26" s="44">
+        <f t="shared" si="5"/>
         <v>46083</v>
       </c>
-      <c r="G26" s="68">
+      <c r="G26" s="50">
         <f>E26+14</f>
         <v>46083</v>
       </c>
       <c r="H26" s="31" t="s">
         <v>59</v>
       </c>
-      <c r="I26" s="69">
-        <f t="shared" si="4"/>
+      <c r="I26" s="51">
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J26" s="31">
@@ -2367,7 +2364,7 @@
     </row>
     <row r="27" spans="1:28" ht="30.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A27" s="21"/>
-      <c r="H27" s="75"/>
+      <c r="H27" s="56"/>
       <c r="I27" s="40"/>
       <c r="J27" s="40"/>
       <c r="K27" s="40"/>
@@ -2391,7 +2388,7 @@
     </row>
     <row r="28" spans="1:28" ht="30" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A28" s="29"/>
-      <c r="H28" s="75"/>
+      <c r="H28" s="56"/>
       <c r="I28" s="40"/>
       <c r="J28" s="40"/>
       <c r="K28" s="40"/>
@@ -2415,7 +2412,7 @@
     </row>
     <row r="29" spans="1:28" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A29" s="21"/>
-      <c r="H29" s="75"/>
+      <c r="H29" s="56"/>
       <c r="I29" s="40"/>
       <c r="J29" s="40"/>
       <c r="K29" s="40"/>
@@ -2439,7 +2436,7 @@
     </row>
     <row r="30" spans="1:28" ht="42.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A30" s="21"/>
-      <c r="H30" s="75"/>
+      <c r="H30" s="56"/>
       <c r="I30" s="40"/>
       <c r="J30" s="40"/>
       <c r="K30" s="40"/>
@@ -2463,7 +2460,7 @@
     </row>
     <row r="31" spans="1:28" ht="17.25" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A31" s="29"/>
-      <c r="H31" s="75"/>
+      <c r="H31" s="56"/>
       <c r="L31" s="33"/>
       <c r="M31" s="33"/>
       <c r="N31" s="33"/>
@@ -2485,7 +2482,7 @@
     <row r="32" spans="1:28" ht="17.25" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A32" s="29"/>
       <c r="G32" s="33"/>
-      <c r="H32" s="75"/>
+      <c r="H32" s="56"/>
       <c r="I32" s="33"/>
       <c r="J32" s="33"/>
       <c r="K32" s="33"/>
@@ -2515,7 +2512,7 @@
       <c r="E33" s="33"/>
       <c r="F33" s="33"/>
       <c r="G33" s="33"/>
-      <c r="H33" s="75"/>
+      <c r="H33" s="56"/>
       <c r="I33" s="33"/>
       <c r="J33" s="33"/>
       <c r="K33" s="33"/>
@@ -2545,7 +2542,7 @@
       <c r="E34" s="33"/>
       <c r="F34" s="33"/>
       <c r="G34" s="33"/>
-      <c r="H34" s="75"/>
+      <c r="H34" s="56"/>
       <c r="I34" s="33"/>
       <c r="J34" s="33"/>
       <c r="K34" s="33"/>
@@ -2575,7 +2572,7 @@
       <c r="E35" s="33"/>
       <c r="F35" s="33"/>
       <c r="G35" s="33"/>
-      <c r="H35" s="75"/>
+      <c r="H35" s="56"/>
       <c r="I35" s="33"/>
       <c r="J35" s="33"/>
       <c r="K35" s="33"/>
@@ -2605,7 +2602,7 @@
       <c r="E36" s="33"/>
       <c r="F36" s="33"/>
       <c r="G36" s="33"/>
-      <c r="H36" s="75"/>
+      <c r="H36" s="56"/>
       <c r="I36" s="33"/>
       <c r="J36" s="33"/>
       <c r="K36" s="33"/>
@@ -2635,7 +2632,7 @@
       <c r="E37" s="33"/>
       <c r="F37" s="33"/>
       <c r="G37" s="33"/>
-      <c r="H37" s="75"/>
+      <c r="H37" s="56"/>
       <c r="I37" s="33"/>
       <c r="J37" s="33"/>
       <c r="K37" s="33"/>
@@ -2664,1714 +2661,1714 @@
       <c r="D38" s="33"/>
       <c r="E38" s="33"/>
       <c r="F38" s="33"/>
-      <c r="H38" s="75"/>
+      <c r="H38" s="56"/>
     </row>
     <row r="39" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H39" s="75"/>
+      <c r="H39" s="56"/>
     </row>
     <row r="40" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H40" s="75"/>
+      <c r="H40" s="56"/>
     </row>
     <row r="41" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H41" s="75"/>
+      <c r="H41" s="56"/>
     </row>
     <row r="42" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H42" s="76"/>
+      <c r="H42" s="57"/>
     </row>
     <row r="43" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H43" s="76"/>
+      <c r="H43" s="57"/>
     </row>
     <row r="44" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H44" s="76"/>
+      <c r="H44" s="57"/>
     </row>
     <row r="45" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H45" s="76"/>
+      <c r="H45" s="57"/>
     </row>
     <row r="46" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H46" s="76"/>
+      <c r="H46" s="57"/>
     </row>
     <row r="47" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H47" s="76"/>
+      <c r="H47" s="57"/>
     </row>
     <row r="48" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H48" s="76"/>
+      <c r="H48" s="57"/>
     </row>
     <row r="49" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H49" s="76"/>
+      <c r="H49" s="57"/>
     </row>
     <row r="50" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H50" s="76"/>
+      <c r="H50" s="57"/>
     </row>
     <row r="51" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H51" s="76"/>
+      <c r="H51" s="57"/>
     </row>
     <row r="52" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H52" s="76"/>
+      <c r="H52" s="57"/>
     </row>
     <row r="53" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H53" s="76"/>
+      <c r="H53" s="57"/>
     </row>
     <row r="54" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H54" s="76"/>
+      <c r="H54" s="57"/>
     </row>
     <row r="55" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H55" s="76"/>
+      <c r="H55" s="57"/>
     </row>
     <row r="56" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H56" s="76"/>
+      <c r="H56" s="57"/>
     </row>
     <row r="57" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H57" s="76"/>
+      <c r="H57" s="57"/>
     </row>
     <row r="58" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H58" s="76"/>
+      <c r="H58" s="57"/>
     </row>
     <row r="59" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H59" s="76"/>
+      <c r="H59" s="57"/>
     </row>
     <row r="60" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H60" s="76"/>
+      <c r="H60" s="57"/>
     </row>
     <row r="61" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H61" s="76"/>
+      <c r="H61" s="57"/>
     </row>
     <row r="62" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H62" s="76"/>
+      <c r="H62" s="57"/>
     </row>
     <row r="63" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H63" s="76"/>
+      <c r="H63" s="57"/>
     </row>
     <row r="64" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H64" s="76"/>
+      <c r="H64" s="57"/>
     </row>
     <row r="65" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H65" s="76"/>
+      <c r="H65" s="57"/>
     </row>
     <row r="66" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H66" s="76"/>
+      <c r="H66" s="57"/>
     </row>
     <row r="67" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H67" s="76"/>
+      <c r="H67" s="57"/>
     </row>
     <row r="68" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H68" s="76"/>
+      <c r="H68" s="57"/>
     </row>
     <row r="69" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H69" s="76"/>
+      <c r="H69" s="57"/>
     </row>
     <row r="70" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H70" s="76"/>
+      <c r="H70" s="57"/>
     </row>
     <row r="71" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H71" s="76"/>
+      <c r="H71" s="57"/>
     </row>
     <row r="72" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H72" s="76"/>
+      <c r="H72" s="57"/>
     </row>
     <row r="73" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H73" s="76"/>
+      <c r="H73" s="57"/>
     </row>
     <row r="74" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H74" s="76"/>
+      <c r="H74" s="57"/>
     </row>
     <row r="75" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H75" s="76"/>
+      <c r="H75" s="57"/>
     </row>
     <row r="76" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H76" s="76"/>
+      <c r="H76" s="57"/>
     </row>
     <row r="77" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H77" s="76"/>
+      <c r="H77" s="57"/>
     </row>
     <row r="78" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H78" s="76"/>
+      <c r="H78" s="57"/>
     </row>
     <row r="79" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H79" s="76"/>
+      <c r="H79" s="57"/>
     </row>
     <row r="80" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H80" s="76"/>
+      <c r="H80" s="57"/>
     </row>
     <row r="81" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H81" s="76"/>
+      <c r="H81" s="57"/>
     </row>
     <row r="82" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H82" s="76"/>
+      <c r="H82" s="57"/>
     </row>
     <row r="83" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H83" s="76"/>
+      <c r="H83" s="57"/>
     </row>
     <row r="84" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H84" s="76"/>
+      <c r="H84" s="57"/>
     </row>
     <row r="85" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H85" s="76"/>
+      <c r="H85" s="57"/>
     </row>
     <row r="86" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H86" s="76"/>
+      <c r="H86" s="57"/>
     </row>
     <row r="87" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H87" s="76"/>
+      <c r="H87" s="57"/>
     </row>
     <row r="88" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H88" s="76"/>
+      <c r="H88" s="57"/>
     </row>
     <row r="89" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H89" s="76"/>
+      <c r="H89" s="57"/>
     </row>
     <row r="90" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H90" s="76"/>
+      <c r="H90" s="57"/>
     </row>
     <row r="91" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H91" s="76"/>
+      <c r="H91" s="57"/>
     </row>
     <row r="92" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H92" s="76"/>
+      <c r="H92" s="57"/>
     </row>
     <row r="93" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H93" s="76"/>
+      <c r="H93" s="57"/>
     </row>
     <row r="94" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H94" s="76"/>
+      <c r="H94" s="57"/>
     </row>
     <row r="95" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H95" s="76"/>
+      <c r="H95" s="57"/>
     </row>
     <row r="96" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H96" s="76"/>
+      <c r="H96" s="57"/>
     </row>
     <row r="97" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H97" s="76"/>
+      <c r="H97" s="57"/>
     </row>
     <row r="98" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H98" s="76"/>
+      <c r="H98" s="57"/>
     </row>
     <row r="99" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H99" s="76"/>
+      <c r="H99" s="57"/>
     </row>
     <row r="100" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H100" s="76"/>
+      <c r="H100" s="57"/>
     </row>
     <row r="101" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H101" s="76"/>
+      <c r="H101" s="57"/>
     </row>
     <row r="102" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H102" s="76"/>
+      <c r="H102" s="57"/>
     </row>
     <row r="103" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H103" s="76"/>
+      <c r="H103" s="57"/>
     </row>
     <row r="104" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H104" s="76"/>
+      <c r="H104" s="57"/>
     </row>
     <row r="105" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H105" s="76"/>
+      <c r="H105" s="57"/>
     </row>
     <row r="106" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H106" s="76"/>
+      <c r="H106" s="57"/>
     </row>
     <row r="107" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H107" s="76"/>
+      <c r="H107" s="57"/>
     </row>
     <row r="108" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H108" s="76"/>
+      <c r="H108" s="57"/>
     </row>
     <row r="109" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H109" s="76"/>
+      <c r="H109" s="57"/>
     </row>
     <row r="110" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H110" s="76"/>
+      <c r="H110" s="57"/>
     </row>
     <row r="111" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H111" s="76"/>
+      <c r="H111" s="57"/>
     </row>
     <row r="112" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H112" s="76"/>
+      <c r="H112" s="57"/>
     </row>
     <row r="113" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H113" s="76"/>
+      <c r="H113" s="57"/>
     </row>
     <row r="114" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H114" s="76"/>
+      <c r="H114" s="57"/>
     </row>
     <row r="115" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H115" s="76"/>
+      <c r="H115" s="57"/>
     </row>
     <row r="116" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H116" s="76"/>
+      <c r="H116" s="57"/>
     </row>
     <row r="117" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H117" s="76"/>
+      <c r="H117" s="57"/>
     </row>
     <row r="118" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H118" s="76"/>
+      <c r="H118" s="57"/>
     </row>
     <row r="119" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H119" s="76"/>
+      <c r="H119" s="57"/>
     </row>
     <row r="120" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H120" s="76"/>
+      <c r="H120" s="57"/>
     </row>
     <row r="121" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H121" s="76"/>
+      <c r="H121" s="57"/>
     </row>
     <row r="122" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H122" s="76"/>
+      <c r="H122" s="57"/>
     </row>
     <row r="123" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H123" s="76"/>
+      <c r="H123" s="57"/>
     </row>
     <row r="124" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H124" s="76"/>
+      <c r="H124" s="57"/>
     </row>
     <row r="125" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H125" s="76"/>
+      <c r="H125" s="57"/>
     </row>
     <row r="126" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H126" s="76"/>
+      <c r="H126" s="57"/>
     </row>
     <row r="127" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H127" s="76"/>
+      <c r="H127" s="57"/>
     </row>
     <row r="128" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H128" s="76"/>
+      <c r="H128" s="57"/>
     </row>
     <row r="129" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H129" s="76"/>
+      <c r="H129" s="57"/>
     </row>
     <row r="130" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H130" s="76"/>
+      <c r="H130" s="57"/>
     </row>
     <row r="131" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H131" s="76"/>
+      <c r="H131" s="57"/>
     </row>
     <row r="132" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H132" s="76"/>
+      <c r="H132" s="57"/>
     </row>
     <row r="133" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H133" s="76"/>
+      <c r="H133" s="57"/>
     </row>
     <row r="134" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H134" s="76"/>
+      <c r="H134" s="57"/>
     </row>
     <row r="135" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H135" s="76"/>
+      <c r="H135" s="57"/>
     </row>
     <row r="136" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H136" s="76"/>
+      <c r="H136" s="57"/>
     </row>
     <row r="137" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H137" s="76"/>
+      <c r="H137" s="57"/>
     </row>
     <row r="138" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H138" s="76"/>
+      <c r="H138" s="57"/>
     </row>
     <row r="139" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H139" s="76"/>
+      <c r="H139" s="57"/>
     </row>
     <row r="140" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H140" s="76"/>
+      <c r="H140" s="57"/>
     </row>
     <row r="141" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H141" s="76"/>
+      <c r="H141" s="57"/>
     </row>
     <row r="142" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H142" s="76"/>
+      <c r="H142" s="57"/>
     </row>
     <row r="143" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H143" s="76"/>
+      <c r="H143" s="57"/>
     </row>
     <row r="144" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H144" s="76"/>
+      <c r="H144" s="57"/>
     </row>
     <row r="145" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H145" s="76"/>
+      <c r="H145" s="57"/>
     </row>
     <row r="146" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H146" s="76"/>
+      <c r="H146" s="57"/>
     </row>
     <row r="147" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H147" s="76"/>
+      <c r="H147" s="57"/>
     </row>
     <row r="148" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H148" s="76"/>
+      <c r="H148" s="57"/>
     </row>
     <row r="149" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H149" s="76"/>
+      <c r="H149" s="57"/>
     </row>
     <row r="150" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H150" s="76"/>
+      <c r="H150" s="57"/>
     </row>
     <row r="151" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H151" s="76"/>
+      <c r="H151" s="57"/>
     </row>
     <row r="152" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H152" s="76"/>
+      <c r="H152" s="57"/>
     </row>
     <row r="153" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H153" s="76"/>
+      <c r="H153" s="57"/>
     </row>
     <row r="154" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H154" s="76"/>
+      <c r="H154" s="57"/>
     </row>
     <row r="155" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H155" s="76"/>
+      <c r="H155" s="57"/>
     </row>
     <row r="156" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H156" s="76"/>
+      <c r="H156" s="57"/>
     </row>
     <row r="157" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H157" s="76"/>
+      <c r="H157" s="57"/>
     </row>
     <row r="158" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H158" s="76"/>
+      <c r="H158" s="57"/>
     </row>
     <row r="159" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H159" s="76"/>
+      <c r="H159" s="57"/>
     </row>
     <row r="160" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H160" s="76"/>
+      <c r="H160" s="57"/>
     </row>
     <row r="161" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H161" s="76"/>
+      <c r="H161" s="57"/>
     </row>
     <row r="162" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H162" s="76"/>
+      <c r="H162" s="57"/>
     </row>
     <row r="163" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H163" s="76"/>
+      <c r="H163" s="57"/>
     </row>
     <row r="164" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H164" s="76"/>
+      <c r="H164" s="57"/>
     </row>
     <row r="165" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H165" s="76"/>
+      <c r="H165" s="57"/>
     </row>
     <row r="166" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H166" s="76"/>
+      <c r="H166" s="57"/>
     </row>
     <row r="167" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H167" s="76"/>
+      <c r="H167" s="57"/>
     </row>
     <row r="168" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H168" s="76"/>
+      <c r="H168" s="57"/>
     </row>
     <row r="169" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H169" s="76"/>
+      <c r="H169" s="57"/>
     </row>
     <row r="170" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H170" s="76"/>
+      <c r="H170" s="57"/>
     </row>
     <row r="171" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H171" s="76"/>
+      <c r="H171" s="57"/>
     </row>
     <row r="172" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H172" s="76"/>
+      <c r="H172" s="57"/>
     </row>
     <row r="173" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H173" s="76"/>
+      <c r="H173" s="57"/>
     </row>
     <row r="174" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H174" s="76"/>
+      <c r="H174" s="57"/>
     </row>
     <row r="175" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H175" s="76"/>
+      <c r="H175" s="57"/>
     </row>
     <row r="176" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H176" s="76"/>
+      <c r="H176" s="57"/>
     </row>
     <row r="177" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H177" s="76"/>
+      <c r="H177" s="57"/>
     </row>
     <row r="178" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H178" s="76"/>
+      <c r="H178" s="57"/>
     </row>
     <row r="179" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H179" s="76"/>
+      <c r="H179" s="57"/>
     </row>
     <row r="180" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H180" s="76"/>
+      <c r="H180" s="57"/>
     </row>
     <row r="181" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H181" s="76"/>
+      <c r="H181" s="57"/>
     </row>
     <row r="182" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H182" s="76"/>
+      <c r="H182" s="57"/>
     </row>
     <row r="183" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H183" s="76"/>
+      <c r="H183" s="57"/>
     </row>
     <row r="184" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H184" s="76"/>
+      <c r="H184" s="57"/>
     </row>
     <row r="185" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H185" s="76"/>
+      <c r="H185" s="57"/>
     </row>
     <row r="186" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H186" s="76"/>
+      <c r="H186" s="57"/>
     </row>
     <row r="187" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H187" s="76"/>
+      <c r="H187" s="57"/>
     </row>
     <row r="188" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H188" s="76"/>
+      <c r="H188" s="57"/>
     </row>
     <row r="189" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H189" s="76"/>
+      <c r="H189" s="57"/>
     </row>
     <row r="190" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H190" s="76"/>
+      <c r="H190" s="57"/>
     </row>
     <row r="191" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H191" s="76"/>
+      <c r="H191" s="57"/>
     </row>
     <row r="192" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H192" s="76"/>
+      <c r="H192" s="57"/>
     </row>
     <row r="193" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H193" s="76"/>
+      <c r="H193" s="57"/>
     </row>
     <row r="194" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H194" s="76"/>
+      <c r="H194" s="57"/>
     </row>
     <row r="195" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H195" s="76"/>
+      <c r="H195" s="57"/>
     </row>
     <row r="196" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H196" s="76"/>
+      <c r="H196" s="57"/>
     </row>
     <row r="197" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H197" s="76"/>
+      <c r="H197" s="57"/>
     </row>
     <row r="198" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H198" s="76"/>
+      <c r="H198" s="57"/>
     </row>
     <row r="199" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H199" s="76"/>
+      <c r="H199" s="57"/>
     </row>
     <row r="200" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H200" s="76"/>
+      <c r="H200" s="57"/>
     </row>
     <row r="201" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H201" s="76"/>
+      <c r="H201" s="57"/>
     </row>
     <row r="202" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H202" s="76"/>
+      <c r="H202" s="57"/>
     </row>
     <row r="203" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H203" s="76"/>
+      <c r="H203" s="57"/>
     </row>
     <row r="204" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H204" s="76"/>
+      <c r="H204" s="57"/>
     </row>
     <row r="205" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H205" s="76"/>
+      <c r="H205" s="57"/>
     </row>
     <row r="206" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H206" s="76"/>
+      <c r="H206" s="57"/>
     </row>
     <row r="207" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H207" s="76"/>
+      <c r="H207" s="57"/>
     </row>
     <row r="208" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H208" s="76"/>
+      <c r="H208" s="57"/>
     </row>
     <row r="209" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H209" s="76"/>
+      <c r="H209" s="57"/>
     </row>
     <row r="210" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H210" s="76"/>
+      <c r="H210" s="57"/>
     </row>
     <row r="211" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H211" s="76"/>
+      <c r="H211" s="57"/>
     </row>
     <row r="212" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H212" s="76"/>
+      <c r="H212" s="57"/>
     </row>
     <row r="213" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H213" s="76"/>
+      <c r="H213" s="57"/>
     </row>
     <row r="214" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H214" s="76"/>
+      <c r="H214" s="57"/>
     </row>
     <row r="215" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H215" s="76"/>
+      <c r="H215" s="57"/>
     </row>
     <row r="216" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H216" s="76"/>
+      <c r="H216" s="57"/>
     </row>
     <row r="217" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H217" s="76"/>
+      <c r="H217" s="57"/>
     </row>
     <row r="218" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H218" s="76"/>
+      <c r="H218" s="57"/>
     </row>
     <row r="219" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H219" s="76"/>
+      <c r="H219" s="57"/>
     </row>
     <row r="220" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H220" s="76"/>
+      <c r="H220" s="57"/>
     </row>
     <row r="221" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H221" s="76"/>
+      <c r="H221" s="57"/>
     </row>
     <row r="222" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H222" s="76"/>
+      <c r="H222" s="57"/>
     </row>
     <row r="223" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H223" s="76"/>
+      <c r="H223" s="57"/>
     </row>
     <row r="224" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H224" s="76"/>
+      <c r="H224" s="57"/>
     </row>
     <row r="225" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H225" s="76"/>
+      <c r="H225" s="57"/>
     </row>
     <row r="226" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H226" s="76"/>
+      <c r="H226" s="57"/>
     </row>
     <row r="227" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H227" s="76"/>
+      <c r="H227" s="57"/>
     </row>
     <row r="228" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H228" s="76"/>
+      <c r="H228" s="57"/>
     </row>
     <row r="229" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H229" s="76"/>
+      <c r="H229" s="57"/>
     </row>
     <row r="230" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H230" s="76"/>
+      <c r="H230" s="57"/>
     </row>
     <row r="231" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H231" s="76"/>
+      <c r="H231" s="57"/>
     </row>
     <row r="232" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H232" s="76"/>
+      <c r="H232" s="57"/>
     </row>
     <row r="233" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H233" s="76"/>
+      <c r="H233" s="57"/>
     </row>
     <row r="234" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H234" s="76"/>
+      <c r="H234" s="57"/>
     </row>
     <row r="235" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H235" s="76"/>
+      <c r="H235" s="57"/>
     </row>
     <row r="236" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H236" s="76"/>
+      <c r="H236" s="57"/>
     </row>
     <row r="237" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H237" s="76"/>
+      <c r="H237" s="57"/>
     </row>
     <row r="238" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H238" s="76"/>
+      <c r="H238" s="57"/>
     </row>
     <row r="239" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H239" s="76"/>
+      <c r="H239" s="57"/>
     </row>
     <row r="240" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H240" s="76"/>
+      <c r="H240" s="57"/>
     </row>
     <row r="241" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H241" s="76"/>
+      <c r="H241" s="57"/>
     </row>
     <row r="242" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H242" s="76"/>
+      <c r="H242" s="57"/>
     </row>
     <row r="243" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H243" s="76"/>
+      <c r="H243" s="57"/>
     </row>
     <row r="244" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H244" s="76"/>
+      <c r="H244" s="57"/>
     </row>
     <row r="245" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H245" s="76"/>
+      <c r="H245" s="57"/>
     </row>
     <row r="246" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H246" s="76"/>
+      <c r="H246" s="57"/>
     </row>
     <row r="247" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H247" s="76"/>
+      <c r="H247" s="57"/>
     </row>
     <row r="248" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H248" s="76"/>
+      <c r="H248" s="57"/>
     </row>
     <row r="249" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H249" s="76"/>
+      <c r="H249" s="57"/>
     </row>
     <row r="250" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H250" s="76"/>
+      <c r="H250" s="57"/>
     </row>
     <row r="251" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H251" s="76"/>
+      <c r="H251" s="57"/>
     </row>
     <row r="252" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H252" s="76"/>
+      <c r="H252" s="57"/>
     </row>
     <row r="253" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H253" s="76"/>
+      <c r="H253" s="57"/>
     </row>
     <row r="254" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H254" s="76"/>
+      <c r="H254" s="57"/>
     </row>
     <row r="255" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H255" s="76"/>
+      <c r="H255" s="57"/>
     </row>
     <row r="256" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H256" s="76"/>
+      <c r="H256" s="57"/>
     </row>
     <row r="257" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H257" s="76"/>
+      <c r="H257" s="57"/>
     </row>
     <row r="258" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H258" s="76"/>
+      <c r="H258" s="57"/>
     </row>
     <row r="259" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H259" s="76"/>
+      <c r="H259" s="57"/>
     </row>
     <row r="260" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H260" s="76"/>
+      <c r="H260" s="57"/>
     </row>
     <row r="261" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H261" s="76"/>
+      <c r="H261" s="57"/>
     </row>
     <row r="262" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H262" s="76"/>
+      <c r="H262" s="57"/>
     </row>
     <row r="263" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H263" s="76"/>
+      <c r="H263" s="57"/>
     </row>
     <row r="264" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H264" s="76"/>
+      <c r="H264" s="57"/>
     </row>
     <row r="265" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H265" s="76"/>
+      <c r="H265" s="57"/>
     </row>
     <row r="266" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H266" s="76"/>
+      <c r="H266" s="57"/>
     </row>
     <row r="267" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H267" s="76"/>
+      <c r="H267" s="57"/>
     </row>
     <row r="268" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H268" s="76"/>
+      <c r="H268" s="57"/>
     </row>
     <row r="269" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H269" s="76"/>
+      <c r="H269" s="57"/>
     </row>
     <row r="270" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H270" s="76"/>
+      <c r="H270" s="57"/>
     </row>
     <row r="271" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H271" s="76"/>
+      <c r="H271" s="57"/>
     </row>
     <row r="272" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H272" s="76"/>
+      <c r="H272" s="57"/>
     </row>
     <row r="273" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H273" s="76"/>
+      <c r="H273" s="57"/>
     </row>
     <row r="274" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H274" s="76"/>
+      <c r="H274" s="57"/>
     </row>
     <row r="275" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H275" s="76"/>
+      <c r="H275" s="57"/>
     </row>
     <row r="276" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H276" s="76"/>
+      <c r="H276" s="57"/>
     </row>
     <row r="277" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H277" s="76"/>
+      <c r="H277" s="57"/>
     </row>
     <row r="278" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H278" s="76"/>
+      <c r="H278" s="57"/>
     </row>
     <row r="279" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H279" s="76"/>
+      <c r="H279" s="57"/>
     </row>
     <row r="280" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H280" s="76"/>
+      <c r="H280" s="57"/>
     </row>
     <row r="281" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H281" s="76"/>
+      <c r="H281" s="57"/>
     </row>
     <row r="282" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H282" s="76"/>
+      <c r="H282" s="57"/>
     </row>
     <row r="283" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H283" s="76"/>
+      <c r="H283" s="57"/>
     </row>
     <row r="284" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H284" s="76"/>
+      <c r="H284" s="57"/>
     </row>
     <row r="285" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H285" s="76"/>
+      <c r="H285" s="57"/>
     </row>
     <row r="286" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H286" s="76"/>
+      <c r="H286" s="57"/>
     </row>
     <row r="287" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H287" s="76"/>
+      <c r="H287" s="57"/>
     </row>
     <row r="288" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H288" s="76"/>
+      <c r="H288" s="57"/>
     </row>
     <row r="289" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H289" s="76"/>
+      <c r="H289" s="57"/>
     </row>
     <row r="290" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H290" s="76"/>
+      <c r="H290" s="57"/>
     </row>
     <row r="291" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H291" s="76"/>
+      <c r="H291" s="57"/>
     </row>
     <row r="292" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H292" s="76"/>
+      <c r="H292" s="57"/>
     </row>
     <row r="293" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H293" s="76"/>
+      <c r="H293" s="57"/>
     </row>
     <row r="294" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H294" s="76"/>
+      <c r="H294" s="57"/>
     </row>
     <row r="295" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H295" s="76"/>
+      <c r="H295" s="57"/>
     </row>
     <row r="296" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H296" s="76"/>
+      <c r="H296" s="57"/>
     </row>
     <row r="297" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H297" s="76"/>
+      <c r="H297" s="57"/>
     </row>
     <row r="298" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H298" s="76"/>
+      <c r="H298" s="57"/>
     </row>
     <row r="299" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H299" s="76"/>
+      <c r="H299" s="57"/>
     </row>
     <row r="300" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H300" s="76"/>
+      <c r="H300" s="57"/>
     </row>
     <row r="301" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H301" s="76"/>
+      <c r="H301" s="57"/>
     </row>
     <row r="302" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H302" s="76"/>
+      <c r="H302" s="57"/>
     </row>
     <row r="303" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H303" s="76"/>
+      <c r="H303" s="57"/>
     </row>
     <row r="304" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H304" s="76"/>
+      <c r="H304" s="57"/>
     </row>
     <row r="305" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H305" s="76"/>
+      <c r="H305" s="57"/>
     </row>
     <row r="306" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H306" s="76"/>
+      <c r="H306" s="57"/>
     </row>
     <row r="307" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H307" s="76"/>
+      <c r="H307" s="57"/>
     </row>
     <row r="308" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H308" s="76"/>
+      <c r="H308" s="57"/>
     </row>
     <row r="309" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H309" s="76"/>
+      <c r="H309" s="57"/>
     </row>
     <row r="310" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H310" s="76"/>
+      <c r="H310" s="57"/>
     </row>
     <row r="311" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H311" s="76"/>
+      <c r="H311" s="57"/>
     </row>
     <row r="312" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H312" s="76"/>
+      <c r="H312" s="57"/>
     </row>
     <row r="313" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H313" s="76"/>
+      <c r="H313" s="57"/>
     </row>
     <row r="314" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H314" s="76"/>
+      <c r="H314" s="57"/>
     </row>
     <row r="315" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H315" s="76"/>
+      <c r="H315" s="57"/>
     </row>
     <row r="316" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H316" s="76"/>
+      <c r="H316" s="57"/>
     </row>
     <row r="317" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H317" s="76"/>
+      <c r="H317" s="57"/>
     </row>
     <row r="318" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H318" s="76"/>
+      <c r="H318" s="57"/>
     </row>
     <row r="319" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H319" s="76"/>
+      <c r="H319" s="57"/>
     </row>
     <row r="320" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H320" s="76"/>
+      <c r="H320" s="57"/>
     </row>
     <row r="321" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H321" s="76"/>
+      <c r="H321" s="57"/>
     </row>
     <row r="322" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H322" s="76"/>
+      <c r="H322" s="57"/>
     </row>
     <row r="323" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H323" s="76"/>
+      <c r="H323" s="57"/>
     </row>
     <row r="324" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H324" s="76"/>
+      <c r="H324" s="57"/>
     </row>
     <row r="325" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H325" s="76"/>
+      <c r="H325" s="57"/>
     </row>
     <row r="326" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H326" s="76"/>
+      <c r="H326" s="57"/>
     </row>
     <row r="327" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H327" s="76"/>
+      <c r="H327" s="57"/>
     </row>
     <row r="328" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H328" s="76"/>
+      <c r="H328" s="57"/>
     </row>
     <row r="329" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H329" s="76"/>
+      <c r="H329" s="57"/>
     </row>
     <row r="330" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H330" s="76"/>
+      <c r="H330" s="57"/>
     </row>
     <row r="331" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H331" s="76"/>
+      <c r="H331" s="57"/>
     </row>
     <row r="332" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H332" s="76"/>
+      <c r="H332" s="57"/>
     </row>
     <row r="333" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H333" s="76"/>
+      <c r="H333" s="57"/>
     </row>
     <row r="334" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H334" s="76"/>
+      <c r="H334" s="57"/>
     </row>
     <row r="335" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H335" s="76"/>
+      <c r="H335" s="57"/>
     </row>
     <row r="336" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H336" s="76"/>
+      <c r="H336" s="57"/>
     </row>
     <row r="337" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H337" s="76"/>
+      <c r="H337" s="57"/>
     </row>
     <row r="338" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H338" s="76"/>
+      <c r="H338" s="57"/>
     </row>
     <row r="339" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H339" s="76"/>
+      <c r="H339" s="57"/>
     </row>
     <row r="340" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H340" s="76"/>
+      <c r="H340" s="57"/>
     </row>
     <row r="341" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H341" s="76"/>
+      <c r="H341" s="57"/>
     </row>
     <row r="342" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H342" s="76"/>
+      <c r="H342" s="57"/>
     </row>
     <row r="343" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H343" s="76"/>
+      <c r="H343" s="57"/>
     </row>
     <row r="344" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H344" s="76"/>
+      <c r="H344" s="57"/>
     </row>
     <row r="345" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H345" s="76"/>
+      <c r="H345" s="57"/>
     </row>
     <row r="346" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H346" s="76"/>
+      <c r="H346" s="57"/>
     </row>
     <row r="347" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H347" s="76"/>
+      <c r="H347" s="57"/>
     </row>
     <row r="348" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H348" s="76"/>
+      <c r="H348" s="57"/>
     </row>
     <row r="349" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H349" s="76"/>
+      <c r="H349" s="57"/>
     </row>
     <row r="350" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H350" s="76"/>
+      <c r="H350" s="57"/>
     </row>
     <row r="351" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H351" s="76"/>
+      <c r="H351" s="57"/>
     </row>
     <row r="352" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H352" s="76"/>
+      <c r="H352" s="57"/>
     </row>
     <row r="353" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H353" s="76"/>
+      <c r="H353" s="57"/>
     </row>
     <row r="354" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H354" s="76"/>
+      <c r="H354" s="57"/>
     </row>
     <row r="355" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H355" s="76"/>
+      <c r="H355" s="57"/>
     </row>
     <row r="356" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H356" s="76"/>
+      <c r="H356" s="57"/>
     </row>
     <row r="357" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H357" s="76"/>
+      <c r="H357" s="57"/>
     </row>
     <row r="358" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H358" s="76"/>
+      <c r="H358" s="57"/>
     </row>
     <row r="359" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H359" s="76"/>
+      <c r="H359" s="57"/>
     </row>
     <row r="360" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H360" s="76"/>
+      <c r="H360" s="57"/>
     </row>
     <row r="361" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H361" s="76"/>
+      <c r="H361" s="57"/>
     </row>
     <row r="362" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H362" s="76"/>
+      <c r="H362" s="57"/>
     </row>
     <row r="363" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H363" s="76"/>
+      <c r="H363" s="57"/>
     </row>
     <row r="364" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H364" s="76"/>
+      <c r="H364" s="57"/>
     </row>
     <row r="365" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H365" s="76"/>
+      <c r="H365" s="57"/>
     </row>
     <row r="366" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H366" s="76"/>
+      <c r="H366" s="57"/>
     </row>
     <row r="367" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H367" s="76"/>
+      <c r="H367" s="57"/>
     </row>
     <row r="368" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H368" s="76"/>
+      <c r="H368" s="57"/>
     </row>
     <row r="369" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H369" s="76"/>
+      <c r="H369" s="57"/>
     </row>
     <row r="370" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H370" s="76"/>
+      <c r="H370" s="57"/>
     </row>
     <row r="371" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H371" s="76"/>
+      <c r="H371" s="57"/>
     </row>
     <row r="372" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H372" s="76"/>
+      <c r="H372" s="57"/>
     </row>
     <row r="373" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H373" s="76"/>
+      <c r="H373" s="57"/>
     </row>
     <row r="374" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H374" s="76"/>
+      <c r="H374" s="57"/>
     </row>
     <row r="375" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H375" s="76"/>
+      <c r="H375" s="57"/>
     </row>
     <row r="376" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H376" s="76"/>
+      <c r="H376" s="57"/>
     </row>
     <row r="377" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H377" s="76"/>
+      <c r="H377" s="57"/>
     </row>
     <row r="378" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H378" s="76"/>
+      <c r="H378" s="57"/>
     </row>
     <row r="379" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H379" s="76"/>
+      <c r="H379" s="57"/>
     </row>
     <row r="380" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H380" s="76"/>
+      <c r="H380" s="57"/>
     </row>
     <row r="381" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H381" s="76"/>
+      <c r="H381" s="57"/>
     </row>
     <row r="382" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H382" s="76"/>
+      <c r="H382" s="57"/>
     </row>
     <row r="383" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H383" s="76"/>
+      <c r="H383" s="57"/>
     </row>
     <row r="384" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H384" s="76"/>
+      <c r="H384" s="57"/>
     </row>
     <row r="385" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H385" s="76"/>
+      <c r="H385" s="57"/>
     </row>
     <row r="386" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H386" s="76"/>
+      <c r="H386" s="57"/>
     </row>
     <row r="387" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H387" s="76"/>
+      <c r="H387" s="57"/>
     </row>
     <row r="388" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H388" s="76"/>
+      <c r="H388" s="57"/>
     </row>
     <row r="389" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H389" s="76"/>
+      <c r="H389" s="57"/>
     </row>
     <row r="390" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H390" s="76"/>
+      <c r="H390" s="57"/>
     </row>
     <row r="391" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H391" s="76"/>
+      <c r="H391" s="57"/>
     </row>
     <row r="392" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H392" s="76"/>
+      <c r="H392" s="57"/>
     </row>
     <row r="393" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H393" s="76"/>
+      <c r="H393" s="57"/>
     </row>
     <row r="394" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H394" s="76"/>
+      <c r="H394" s="57"/>
     </row>
     <row r="395" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H395" s="76"/>
+      <c r="H395" s="57"/>
     </row>
     <row r="396" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H396" s="76"/>
+      <c r="H396" s="57"/>
     </row>
     <row r="397" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H397" s="76"/>
+      <c r="H397" s="57"/>
     </row>
     <row r="398" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H398" s="76"/>
+      <c r="H398" s="57"/>
     </row>
     <row r="399" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H399" s="76"/>
+      <c r="H399" s="57"/>
     </row>
     <row r="400" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H400" s="76"/>
+      <c r="H400" s="57"/>
     </row>
     <row r="401" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H401" s="76"/>
+      <c r="H401" s="57"/>
     </row>
     <row r="402" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H402" s="76"/>
+      <c r="H402" s="57"/>
     </row>
     <row r="403" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H403" s="76"/>
+      <c r="H403" s="57"/>
     </row>
     <row r="404" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H404" s="76"/>
+      <c r="H404" s="57"/>
     </row>
     <row r="405" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H405" s="76"/>
+      <c r="H405" s="57"/>
     </row>
     <row r="406" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H406" s="76"/>
+      <c r="H406" s="57"/>
     </row>
     <row r="407" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H407" s="76"/>
+      <c r="H407" s="57"/>
     </row>
     <row r="408" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H408" s="76"/>
+      <c r="H408" s="57"/>
     </row>
     <row r="409" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H409" s="76"/>
+      <c r="H409" s="57"/>
     </row>
     <row r="410" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H410" s="76"/>
+      <c r="H410" s="57"/>
     </row>
     <row r="411" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H411" s="76"/>
+      <c r="H411" s="57"/>
     </row>
     <row r="412" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H412" s="76"/>
+      <c r="H412" s="57"/>
     </row>
     <row r="413" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H413" s="76"/>
+      <c r="H413" s="57"/>
     </row>
     <row r="414" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H414" s="76"/>
+      <c r="H414" s="57"/>
     </row>
     <row r="415" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H415" s="76"/>
+      <c r="H415" s="57"/>
     </row>
     <row r="416" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H416" s="76"/>
+      <c r="H416" s="57"/>
     </row>
     <row r="417" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H417" s="76"/>
+      <c r="H417" s="57"/>
     </row>
     <row r="418" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H418" s="76"/>
+      <c r="H418" s="57"/>
     </row>
     <row r="419" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H419" s="76"/>
+      <c r="H419" s="57"/>
     </row>
     <row r="420" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H420" s="76"/>
+      <c r="H420" s="57"/>
     </row>
     <row r="421" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H421" s="76"/>
+      <c r="H421" s="57"/>
     </row>
     <row r="422" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H422" s="76"/>
+      <c r="H422" s="57"/>
     </row>
     <row r="423" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H423" s="76"/>
+      <c r="H423" s="57"/>
     </row>
     <row r="424" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H424" s="76"/>
+      <c r="H424" s="57"/>
     </row>
     <row r="425" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H425" s="76"/>
+      <c r="H425" s="57"/>
     </row>
     <row r="426" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H426" s="76"/>
+      <c r="H426" s="57"/>
     </row>
     <row r="427" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H427" s="76"/>
+      <c r="H427" s="57"/>
     </row>
     <row r="428" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H428" s="76"/>
+      <c r="H428" s="57"/>
     </row>
     <row r="429" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H429" s="76"/>
+      <c r="H429" s="57"/>
     </row>
     <row r="430" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H430" s="76"/>
+      <c r="H430" s="57"/>
     </row>
     <row r="431" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H431" s="76"/>
+      <c r="H431" s="57"/>
     </row>
     <row r="432" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H432" s="76"/>
+      <c r="H432" s="57"/>
     </row>
     <row r="433" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H433" s="76"/>
+      <c r="H433" s="57"/>
     </row>
     <row r="434" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H434" s="76"/>
+      <c r="H434" s="57"/>
     </row>
     <row r="435" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H435" s="76"/>
+      <c r="H435" s="57"/>
     </row>
     <row r="436" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H436" s="76"/>
+      <c r="H436" s="57"/>
     </row>
     <row r="437" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H437" s="76"/>
+      <c r="H437" s="57"/>
     </row>
     <row r="438" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H438" s="76"/>
+      <c r="H438" s="57"/>
     </row>
     <row r="439" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H439" s="76"/>
+      <c r="H439" s="57"/>
     </row>
     <row r="440" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H440" s="76"/>
+      <c r="H440" s="57"/>
     </row>
     <row r="441" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H441" s="76"/>
+      <c r="H441" s="57"/>
     </row>
     <row r="442" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H442" s="76"/>
+      <c r="H442" s="57"/>
     </row>
     <row r="443" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H443" s="76"/>
+      <c r="H443" s="57"/>
     </row>
     <row r="444" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H444" s="76"/>
+      <c r="H444" s="57"/>
     </row>
     <row r="445" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H445" s="76"/>
+      <c r="H445" s="57"/>
     </row>
     <row r="446" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H446" s="76"/>
+      <c r="H446" s="57"/>
     </row>
     <row r="447" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H447" s="76"/>
+      <c r="H447" s="57"/>
     </row>
     <row r="448" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H448" s="76"/>
+      <c r="H448" s="57"/>
     </row>
     <row r="449" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H449" s="76"/>
+      <c r="H449" s="57"/>
     </row>
     <row r="450" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H450" s="76"/>
+      <c r="H450" s="57"/>
     </row>
     <row r="451" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H451" s="76"/>
+      <c r="H451" s="57"/>
     </row>
     <row r="452" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H452" s="76"/>
+      <c r="H452" s="57"/>
     </row>
     <row r="453" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H453" s="76"/>
+      <c r="H453" s="57"/>
     </row>
     <row r="454" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H454" s="76"/>
+      <c r="H454" s="57"/>
     </row>
     <row r="455" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H455" s="76"/>
+      <c r="H455" s="57"/>
     </row>
     <row r="456" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H456" s="76"/>
+      <c r="H456" s="57"/>
     </row>
     <row r="457" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H457" s="76"/>
+      <c r="H457" s="57"/>
     </row>
     <row r="458" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H458" s="76"/>
+      <c r="H458" s="57"/>
     </row>
     <row r="459" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H459" s="76"/>
+      <c r="H459" s="57"/>
     </row>
     <row r="460" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H460" s="76"/>
+      <c r="H460" s="57"/>
     </row>
     <row r="461" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H461" s="76"/>
+      <c r="H461" s="57"/>
     </row>
     <row r="462" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H462" s="76"/>
+      <c r="H462" s="57"/>
     </row>
     <row r="463" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H463" s="76"/>
+      <c r="H463" s="57"/>
     </row>
     <row r="464" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H464" s="76"/>
+      <c r="H464" s="57"/>
     </row>
     <row r="465" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H465" s="76"/>
+      <c r="H465" s="57"/>
     </row>
     <row r="466" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H466" s="76"/>
+      <c r="H466" s="57"/>
     </row>
     <row r="467" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H467" s="76"/>
+      <c r="H467" s="57"/>
     </row>
     <row r="468" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H468" s="76"/>
+      <c r="H468" s="57"/>
     </row>
     <row r="469" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H469" s="76"/>
+      <c r="H469" s="57"/>
     </row>
     <row r="470" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H470" s="76"/>
+      <c r="H470" s="57"/>
     </row>
     <row r="471" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H471" s="76"/>
+      <c r="H471" s="57"/>
     </row>
     <row r="472" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H472" s="76"/>
+      <c r="H472" s="57"/>
     </row>
     <row r="473" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H473" s="76"/>
+      <c r="H473" s="57"/>
     </row>
     <row r="474" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H474" s="76"/>
+      <c r="H474" s="57"/>
     </row>
     <row r="475" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H475" s="76"/>
+      <c r="H475" s="57"/>
     </row>
     <row r="476" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H476" s="76"/>
+      <c r="H476" s="57"/>
     </row>
     <row r="477" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H477" s="76"/>
+      <c r="H477" s="57"/>
     </row>
     <row r="478" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H478" s="76"/>
+      <c r="H478" s="57"/>
     </row>
     <row r="479" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H479" s="76"/>
+      <c r="H479" s="57"/>
     </row>
     <row r="480" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H480" s="76"/>
+      <c r="H480" s="57"/>
     </row>
     <row r="481" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H481" s="76"/>
+      <c r="H481" s="57"/>
     </row>
     <row r="482" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H482" s="76"/>
+      <c r="H482" s="57"/>
     </row>
     <row r="483" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H483" s="76"/>
+      <c r="H483" s="57"/>
     </row>
     <row r="484" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H484" s="76"/>
+      <c r="H484" s="57"/>
     </row>
     <row r="485" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H485" s="76"/>
+      <c r="H485" s="57"/>
     </row>
     <row r="486" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H486" s="76"/>
+      <c r="H486" s="57"/>
     </row>
     <row r="487" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H487" s="76"/>
+      <c r="H487" s="57"/>
     </row>
     <row r="488" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H488" s="76"/>
+      <c r="H488" s="57"/>
     </row>
     <row r="489" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H489" s="76"/>
+      <c r="H489" s="57"/>
     </row>
     <row r="490" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H490" s="76"/>
+      <c r="H490" s="57"/>
     </row>
     <row r="491" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H491" s="76"/>
+      <c r="H491" s="57"/>
     </row>
     <row r="492" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H492" s="76"/>
+      <c r="H492" s="57"/>
     </row>
     <row r="493" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H493" s="76"/>
+      <c r="H493" s="57"/>
     </row>
     <row r="494" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H494" s="76"/>
+      <c r="H494" s="57"/>
     </row>
     <row r="495" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H495" s="76"/>
+      <c r="H495" s="57"/>
     </row>
     <row r="496" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H496" s="76"/>
+      <c r="H496" s="57"/>
     </row>
     <row r="497" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H497" s="76"/>
+      <c r="H497" s="57"/>
     </row>
     <row r="498" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H498" s="76"/>
+      <c r="H498" s="57"/>
     </row>
     <row r="499" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H499" s="76"/>
+      <c r="H499" s="57"/>
     </row>
     <row r="500" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H500" s="76"/>
+      <c r="H500" s="57"/>
     </row>
     <row r="501" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H501" s="76"/>
+      <c r="H501" s="57"/>
     </row>
     <row r="502" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H502" s="76"/>
+      <c r="H502" s="57"/>
     </row>
     <row r="503" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H503" s="76"/>
+      <c r="H503" s="57"/>
     </row>
     <row r="504" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H504" s="76"/>
+      <c r="H504" s="57"/>
     </row>
     <row r="505" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H505" s="76"/>
+      <c r="H505" s="57"/>
     </row>
     <row r="506" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H506" s="76"/>
+      <c r="H506" s="57"/>
     </row>
     <row r="507" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H507" s="76"/>
+      <c r="H507" s="57"/>
     </row>
     <row r="508" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H508" s="76"/>
+      <c r="H508" s="57"/>
     </row>
     <row r="509" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H509" s="76"/>
+      <c r="H509" s="57"/>
     </row>
     <row r="510" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H510" s="76"/>
+      <c r="H510" s="57"/>
     </row>
     <row r="511" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H511" s="76"/>
+      <c r="H511" s="57"/>
     </row>
     <row r="512" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H512" s="76"/>
+      <c r="H512" s="57"/>
     </row>
     <row r="513" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H513" s="76"/>
+      <c r="H513" s="57"/>
     </row>
     <row r="514" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H514" s="76"/>
+      <c r="H514" s="57"/>
     </row>
     <row r="515" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H515" s="76"/>
+      <c r="H515" s="57"/>
     </row>
     <row r="516" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H516" s="76"/>
+      <c r="H516" s="57"/>
     </row>
     <row r="517" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H517" s="76"/>
+      <c r="H517" s="57"/>
     </row>
     <row r="518" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H518" s="76"/>
+      <c r="H518" s="57"/>
     </row>
     <row r="519" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H519" s="76"/>
+      <c r="H519" s="57"/>
     </row>
     <row r="520" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H520" s="76"/>
+      <c r="H520" s="57"/>
     </row>
     <row r="521" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H521" s="76"/>
+      <c r="H521" s="57"/>
     </row>
     <row r="522" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H522" s="76"/>
+      <c r="H522" s="57"/>
     </row>
     <row r="523" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H523" s="76"/>
+      <c r="H523" s="57"/>
     </row>
     <row r="524" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H524" s="76"/>
+      <c r="H524" s="57"/>
     </row>
     <row r="525" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H525" s="76"/>
+      <c r="H525" s="57"/>
     </row>
     <row r="526" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H526" s="76"/>
+      <c r="H526" s="57"/>
     </row>
     <row r="527" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H527" s="76"/>
+      <c r="H527" s="57"/>
     </row>
     <row r="528" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H528" s="76"/>
+      <c r="H528" s="57"/>
     </row>
     <row r="529" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H529" s="76"/>
+      <c r="H529" s="57"/>
     </row>
     <row r="530" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H530" s="76"/>
+      <c r="H530" s="57"/>
     </row>
     <row r="531" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H531" s="76"/>
+      <c r="H531" s="57"/>
     </row>
     <row r="532" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H532" s="76"/>
+      <c r="H532" s="57"/>
     </row>
     <row r="533" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H533" s="76"/>
+      <c r="H533" s="57"/>
     </row>
     <row r="534" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H534" s="76"/>
+      <c r="H534" s="57"/>
     </row>
     <row r="535" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H535" s="76"/>
+      <c r="H535" s="57"/>
     </row>
     <row r="536" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H536" s="76"/>
+      <c r="H536" s="57"/>
     </row>
     <row r="537" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H537" s="76"/>
+      <c r="H537" s="57"/>
     </row>
     <row r="538" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H538" s="76"/>
+      <c r="H538" s="57"/>
     </row>
     <row r="539" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H539" s="76"/>
+      <c r="H539" s="57"/>
     </row>
     <row r="540" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H540" s="76"/>
+      <c r="H540" s="57"/>
     </row>
     <row r="541" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H541" s="76"/>
+      <c r="H541" s="57"/>
     </row>
     <row r="542" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H542" s="76"/>
+      <c r="H542" s="57"/>
     </row>
     <row r="543" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H543" s="76"/>
+      <c r="H543" s="57"/>
     </row>
     <row r="544" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H544" s="76"/>
+      <c r="H544" s="57"/>
     </row>
     <row r="545" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H545" s="76"/>
+      <c r="H545" s="57"/>
     </row>
     <row r="546" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H546" s="76"/>
+      <c r="H546" s="57"/>
     </row>
     <row r="547" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H547" s="76"/>
+      <c r="H547" s="57"/>
     </row>
     <row r="548" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H548" s="76"/>
+      <c r="H548" s="57"/>
     </row>
     <row r="549" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H549" s="76"/>
+      <c r="H549" s="57"/>
     </row>
     <row r="550" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H550" s="76"/>
+      <c r="H550" s="57"/>
     </row>
     <row r="551" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H551" s="76"/>
+      <c r="H551" s="57"/>
     </row>
     <row r="552" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H552" s="76"/>
+      <c r="H552" s="57"/>
     </row>
     <row r="553" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H553" s="76"/>
+      <c r="H553" s="57"/>
     </row>
     <row r="554" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H554" s="76"/>
+      <c r="H554" s="57"/>
     </row>
     <row r="555" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H555" s="76"/>
+      <c r="H555" s="57"/>
     </row>
     <row r="556" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H556" s="76"/>
+      <c r="H556" s="57"/>
     </row>
     <row r="557" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H557" s="76"/>
+      <c r="H557" s="57"/>
     </row>
     <row r="558" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H558" s="76"/>
+      <c r="H558" s="57"/>
     </row>
     <row r="559" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H559" s="76"/>
+      <c r="H559" s="57"/>
     </row>
     <row r="560" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H560" s="76"/>
+      <c r="H560" s="57"/>
     </row>
     <row r="561" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H561" s="76"/>
+      <c r="H561" s="57"/>
     </row>
     <row r="562" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H562" s="76"/>
+      <c r="H562" s="57"/>
     </row>
     <row r="563" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H563" s="76"/>
+      <c r="H563" s="57"/>
     </row>
     <row r="564" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H564" s="76"/>
+      <c r="H564" s="57"/>
     </row>
     <row r="565" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H565" s="76"/>
+      <c r="H565" s="57"/>
     </row>
     <row r="566" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H566" s="76"/>
+      <c r="H566" s="57"/>
     </row>
     <row r="567" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H567" s="76"/>
+      <c r="H567" s="57"/>
     </row>
     <row r="568" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H568" s="76"/>
+      <c r="H568" s="57"/>
     </row>
     <row r="569" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H569" s="76"/>
+      <c r="H569" s="57"/>
     </row>
     <row r="570" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H570" s="76"/>
+      <c r="H570" s="57"/>
     </row>
     <row r="571" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H571" s="76"/>
+      <c r="H571" s="57"/>
     </row>
     <row r="572" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H572" s="76"/>
+      <c r="H572" s="57"/>
     </row>
     <row r="573" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H573" s="76"/>
+      <c r="H573" s="57"/>
     </row>
     <row r="574" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H574" s="76"/>
+      <c r="H574" s="57"/>
     </row>
     <row r="575" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H575" s="76"/>
+      <c r="H575" s="57"/>
     </row>
     <row r="576" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H576" s="76"/>
+      <c r="H576" s="57"/>
     </row>
     <row r="577" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H577" s="76"/>
+      <c r="H577" s="57"/>
     </row>
     <row r="578" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H578" s="76"/>
+      <c r="H578" s="57"/>
     </row>
     <row r="579" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H579" s="76"/>
+      <c r="H579" s="57"/>
     </row>
     <row r="580" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H580" s="76"/>
+      <c r="H580" s="57"/>
     </row>
     <row r="581" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H581" s="76"/>
+      <c r="H581" s="57"/>
     </row>
     <row r="582" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H582" s="76"/>
+      <c r="H582" s="57"/>
     </row>
     <row r="583" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H583" s="76"/>
+      <c r="H583" s="57"/>
     </row>
     <row r="584" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H584" s="76"/>
+      <c r="H584" s="57"/>
     </row>
     <row r="585" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H585" s="76"/>
+      <c r="H585" s="57"/>
     </row>
     <row r="586" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H586" s="76"/>
+      <c r="H586" s="57"/>
     </row>
     <row r="587" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H587" s="76"/>
+      <c r="H587" s="57"/>
     </row>
     <row r="588" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H588" s="76"/>
+      <c r="H588" s="57"/>
     </row>
     <row r="589" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H589" s="76"/>
+      <c r="H589" s="57"/>
     </row>
     <row r="590" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H590" s="76"/>
+      <c r="H590" s="57"/>
     </row>
     <row r="591" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H591" s="76"/>
+      <c r="H591" s="57"/>
     </row>
     <row r="592" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H592" s="76"/>
+      <c r="H592" s="57"/>
     </row>
     <row r="593" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H593" s="76"/>
+      <c r="H593" s="57"/>
     </row>
     <row r="594" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H594" s="76"/>
+      <c r="H594" s="57"/>
     </row>
     <row r="595" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H595" s="76"/>
+      <c r="H595" s="57"/>
     </row>
     <row r="596" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H596" s="76"/>
+      <c r="H596" s="57"/>
     </row>
     <row r="597" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H597" s="76"/>
+      <c r="H597" s="57"/>
     </row>
     <row r="598" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H598" s="76"/>
+      <c r="H598" s="57"/>
     </row>
     <row r="599" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H599" s="76"/>
+      <c r="H599" s="57"/>
     </row>
     <row r="600" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H600" s="76"/>
+      <c r="H600" s="57"/>
     </row>
     <row r="601" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H601" s="76"/>
+      <c r="H601" s="57"/>
     </row>
     <row r="602" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H602" s="76"/>
+      <c r="H602" s="57"/>
     </row>
     <row r="603" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H603" s="76"/>
+      <c r="H603" s="57"/>
     </row>
     <row r="604" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H604" s="76"/>
+      <c r="H604" s="57"/>
     </row>
     <row r="605" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H605" s="76"/>
+      <c r="H605" s="57"/>
     </row>
     <row r="606" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H606" s="76"/>
+      <c r="H606" s="57"/>
     </row>
     <row r="607" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H607" s="74"/>
+      <c r="H607" s="55"/>
     </row>
     <row r="608" spans="8:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="609" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -4726,20 +4723,6 @@
     <row r="958" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="26">
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="L4:X4"/>
-    <mergeCell ref="D6:O6"/>
-    <mergeCell ref="D4:H4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="D5:H5"/>
-    <mergeCell ref="J5:K5"/>
-    <mergeCell ref="B2:K2"/>
-    <mergeCell ref="L2:AA2"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="D3:K3"/>
-    <mergeCell ref="L3:T3"/>
-    <mergeCell ref="U3:AA3"/>
     <mergeCell ref="B8:B10"/>
     <mergeCell ref="C8:C10"/>
     <mergeCell ref="D8:D10"/>
@@ -4752,6 +4735,20 @@
     <mergeCell ref="I8:I10"/>
     <mergeCell ref="J8:J10"/>
     <mergeCell ref="K8:K10"/>
+    <mergeCell ref="B2:K2"/>
+    <mergeCell ref="L2:AA2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="D3:K3"/>
+    <mergeCell ref="L3:T3"/>
+    <mergeCell ref="U3:AA3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="L4:X4"/>
+    <mergeCell ref="D6:O6"/>
+    <mergeCell ref="D4:H4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="D5:H5"/>
+    <mergeCell ref="J5:K5"/>
   </mergeCells>
   <phoneticPr fontId="23" type="noConversion"/>
   <conditionalFormatting sqref="L10:AA10">

</xml_diff>